<commit_message>
Explicación breve de los cambios realizados
</commit_message>
<xml_diff>
--- a/facturas/facturas_con_tasa_BCV_CORREGIDO.xlsx
+++ b/facturas/facturas_con_tasa_BCV_CORREGIDO.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jhonny\Desktop\creditos\facturas\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/DB0E4EA3DEA0B523/Desktop/creditos/facturas/"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="11_21082202B7D33F80DDCD1AFB2B819177F2CB411B" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12450"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FACT CARACAS" sheetId="1" r:id="rId1"/>
@@ -18,7 +19,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'FACT CARACAS'!$B$1:$BO$131</definedName>
   </definedNames>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -674,13 +675,13 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="5">
-    <numFmt numFmtId="164" formatCode="_-&quot;XDR&quot;* #,##0.00_-;\-&quot;XDR&quot;* #,##0.00_-;_-&quot;XDR&quot;* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="165" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="166" formatCode="#,##0.00;[Red]#,##0.00"/>
-    <numFmt numFmtId="167" formatCode="#,##0.00_ ;\-#,##0.00\ "/>
-    <numFmt numFmtId="168" formatCode="0.00_ ;\-0.00\ "/>
+    <numFmt numFmtId="44" formatCode="_-&quot;XDR&quot;* #,##0.00_-;\-&quot;XDR&quot;* #,##0.00_-;_-&quot;XDR&quot;* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="#,##0.00;[Red]#,##0.00"/>
+    <numFmt numFmtId="165" formatCode="#,##0.00_ ;\-#,##0.00\ "/>
+    <numFmt numFmtId="166" formatCode="0.00_ ;\-0.00\ "/>
   </numFmts>
   <fonts count="11" x14ac:knownFonts="1">
     <font>
@@ -914,10 +915,10 @@
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0"/>
+    <xf numFmtId="43" fontId="6" fillId="0" borderId="0"/>
+    <xf numFmtId="44" fontId="6" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="145">
+  <cellXfs count="141">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="4" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -1090,22 +1091,22 @@
     <xf numFmtId="4" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="2" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="1" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="2" borderId="1" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="6" fillId="2" borderId="1" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="6" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="2" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1123,7 +1124,7 @@
     <xf numFmtId="4" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1139,7 +1140,7 @@
     <xf numFmtId="1" fontId="7" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="3" fillId="7" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1230,13 +1231,7 @@
     <xf numFmtId="4" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1248,9 +1243,6 @@
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="7" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1279,7 +1271,7 @@
     </xf>
     <xf numFmtId="4" fontId="1" fillId="9" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1298,14 +1290,11 @@
     <xf numFmtId="1" fontId="7" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" shrinkToFit="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1339,10 +1328,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1641,59 +1626,59 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <tabColor theme="7"/>
   </sheetPr>
   <dimension ref="A1:BO152"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="4" style="42" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="9.5703125" style="117" customWidth="1"/>
-    <col min="3" max="3" width="40.5703125" style="58" customWidth="1"/>
-    <col min="4" max="4" width="13.42578125" style="7" customWidth="1"/>
-    <col min="5" max="5" width="17.5703125" style="7" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.5703125" style="7" customWidth="1"/>
+    <col min="2" max="2" width="9.5546875" style="42" customWidth="1"/>
+    <col min="3" max="3" width="40.5546875" style="58" customWidth="1"/>
+    <col min="4" max="4" width="13.44140625" style="7" customWidth="1"/>
+    <col min="5" max="5" width="17.5546875" style="7" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.5546875" style="7" customWidth="1"/>
     <col min="7" max="7" width="20" style="42" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" style="42" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.5703125" style="42" customWidth="1"/>
-    <col min="10" max="11" width="14.7109375" style="32" customWidth="1"/>
-    <col min="12" max="12" width="16.28515625" style="7" customWidth="1"/>
-    <col min="13" max="13" width="11.42578125" style="42" customWidth="1"/>
-    <col min="14" max="14" width="11.28515625" style="58" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="11.28515625" style="59" customWidth="1"/>
-    <col min="16" max="16" width="23.5703125" style="58" customWidth="1"/>
-    <col min="17" max="17" width="14.28515625" style="59" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="16.140625" style="42" customWidth="1"/>
-    <col min="19" max="19" width="12.28515625" style="42" customWidth="1"/>
-    <col min="20" max="20" width="11.28515625" style="7" customWidth="1"/>
-    <col min="21" max="21" width="12.28515625" style="42" customWidth="1"/>
-    <col min="22" max="22" width="12.42578125" style="59" customWidth="1"/>
-    <col min="23" max="23" width="11.5703125" style="58" customWidth="1"/>
-    <col min="24" max="24" width="15.28515625" style="42" customWidth="1"/>
-    <col min="25" max="25" width="11.28515625" style="59" customWidth="1"/>
-    <col min="26" max="26" width="15.28515625" style="42" customWidth="1"/>
-    <col min="27" max="29" width="11.42578125" style="58" customWidth="1"/>
-    <col min="30" max="30" width="11.28515625" style="59" customWidth="1"/>
-    <col min="31" max="34" width="11.42578125" style="58" customWidth="1"/>
-    <col min="35" max="35" width="11.28515625" style="7" customWidth="1"/>
-    <col min="36" max="39" width="11.42578125" style="58" customWidth="1"/>
-    <col min="40" max="40" width="11.28515625" style="59" customWidth="1"/>
-    <col min="41" max="44" width="11.42578125" style="58" customWidth="1"/>
-    <col min="45" max="45" width="11.28515625" style="59" customWidth="1"/>
-    <col min="46" max="49" width="11.42578125" style="58" customWidth="1"/>
-    <col min="50" max="50" width="11.28515625" style="59" customWidth="1"/>
-    <col min="51" max="54" width="11.42578125" style="58" customWidth="1"/>
-    <col min="55" max="55" width="11.28515625" style="59" customWidth="1"/>
-    <col min="56" max="56" width="11.42578125" style="58" customWidth="1"/>
-    <col min="57" max="59" width="11.42578125" style="58"/>
-    <col min="60" max="61" width="11.42578125" style="58" customWidth="1"/>
-    <col min="62" max="64" width="11.42578125" style="58"/>
-    <col min="65" max="66" width="11.42578125" style="58" customWidth="1"/>
-    <col min="67" max="16384" width="11.42578125" style="58"/>
+    <col min="8" max="8" width="10.109375" style="42" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.5546875" style="42" customWidth="1"/>
+    <col min="10" max="11" width="14.6640625" style="32" customWidth="1"/>
+    <col min="12" max="12" width="16.33203125" style="7" customWidth="1"/>
+    <col min="13" max="13" width="11.44140625" style="42" customWidth="1"/>
+    <col min="14" max="14" width="11.33203125" style="58" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="11.33203125" style="59" customWidth="1"/>
+    <col min="16" max="16" width="23.5546875" style="58" customWidth="1"/>
+    <col min="17" max="17" width="14.33203125" style="59" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="16.109375" style="42" customWidth="1"/>
+    <col min="19" max="19" width="12.33203125" style="42" customWidth="1"/>
+    <col min="20" max="20" width="11.33203125" style="7" customWidth="1"/>
+    <col min="21" max="21" width="12.33203125" style="42" customWidth="1"/>
+    <col min="22" max="22" width="12.44140625" style="59" customWidth="1"/>
+    <col min="23" max="23" width="11.5546875" style="58" customWidth="1"/>
+    <col min="24" max="24" width="15.33203125" style="42" customWidth="1"/>
+    <col min="25" max="25" width="11.33203125" style="59" customWidth="1"/>
+    <col min="26" max="26" width="15.33203125" style="42" customWidth="1"/>
+    <col min="27" max="29" width="11.44140625" style="58" customWidth="1"/>
+    <col min="30" max="30" width="11.33203125" style="59" customWidth="1"/>
+    <col min="31" max="34" width="11.44140625" style="58" customWidth="1"/>
+    <col min="35" max="35" width="11.33203125" style="7" customWidth="1"/>
+    <col min="36" max="39" width="11.44140625" style="58" customWidth="1"/>
+    <col min="40" max="40" width="11.33203125" style="59" customWidth="1"/>
+    <col min="41" max="44" width="11.44140625" style="58" customWidth="1"/>
+    <col min="45" max="45" width="11.33203125" style="59" customWidth="1"/>
+    <col min="46" max="49" width="11.44140625" style="58" customWidth="1"/>
+    <col min="50" max="50" width="11.33203125" style="59" customWidth="1"/>
+    <col min="51" max="54" width="11.44140625" style="58" customWidth="1"/>
+    <col min="55" max="55" width="11.33203125" style="59" customWidth="1"/>
+    <col min="56" max="56" width="11.44140625" style="58" customWidth="1"/>
+    <col min="57" max="59" width="11.44140625" style="58"/>
+    <col min="60" max="61" width="11.44140625" style="58" customWidth="1"/>
+    <col min="62" max="64" width="11.44140625" style="58"/>
+    <col min="65" max="66" width="11.44140625" style="58" customWidth="1"/>
+    <col min="67" max="16384" width="11.44140625" style="58"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:67" s="10" customFormat="1" ht="40.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:67" s="10" customFormat="1" ht="40.200000000000003" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="62" t="s">
         <v>0</v>
       </c>
@@ -1894,11 +1879,11 @@
       </c>
       <c r="BO1" s="57"/>
     </row>
-    <row r="2" spans="1:67" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:67" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="42">
         <v>1</v>
       </c>
-      <c r="B2" s="116">
+      <c r="B2" s="2">
         <v>7693</v>
       </c>
       <c r="C2" s="53" t="s">
@@ -2028,11 +2013,11 @@
       <c r="BC2" s="51"/>
       <c r="BD2" s="51"/>
     </row>
-    <row r="3" spans="1:67" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:67" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A3" s="42">
         <v>2</v>
       </c>
-      <c r="B3" s="116">
+      <c r="B3" s="2">
         <v>7965</v>
       </c>
       <c r="C3" s="53" t="s">
@@ -2046,7 +2031,7 @@
         <v>222.16008974384832</v>
       </c>
       <c r="F3" s="51">
-        <f t="shared" ref="F3:F66" si="2">E3/4</f>
+        <f t="shared" ref="F3:F65" si="2">E3/4</f>
         <v>55.540022435962079</v>
       </c>
       <c r="G3" s="50">
@@ -2181,11 +2166,11 @@
       <c r="BC3" s="14"/>
       <c r="BD3" s="51"/>
     </row>
-    <row r="4" spans="1:67" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:67" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="42">
         <v>3</v>
       </c>
-      <c r="B4" s="116">
+      <c r="B4" s="2">
         <v>8526</v>
       </c>
       <c r="C4" s="11" t="s">
@@ -2284,11 +2269,11 @@
       <c r="BC4" s="63"/>
       <c r="BD4" s="51"/>
     </row>
-    <row r="5" spans="1:67" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:67" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="42">
         <v>4</v>
       </c>
-      <c r="B5" s="116">
+      <c r="B5" s="2">
         <v>9642</v>
       </c>
       <c r="C5" s="11" t="s">
@@ -2298,7 +2283,7 @@
         <v>12741.43</v>
       </c>
       <c r="E5" s="51">
-        <f t="shared" ref="E4:E67" si="9">D5/H5</f>
+        <f t="shared" ref="E5:E67" si="9">D5/H5</f>
         <v>131.87756428568471</v>
       </c>
       <c r="F5" s="51">
@@ -2393,11 +2378,11 @@
       <c r="BC5" s="51"/>
       <c r="BD5" s="51"/>
     </row>
-    <row r="6" spans="1:67" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:67" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="42">
         <v>5</v>
       </c>
-      <c r="B6" s="116">
+      <c r="B6" s="2">
         <v>9716</v>
       </c>
       <c r="C6" s="53" t="s">
@@ -2558,11 +2543,11 @@
       <c r="BC6" s="51"/>
       <c r="BD6" s="51"/>
     </row>
-    <row r="7" spans="1:67" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:67" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A7" s="42">
         <v>6</v>
       </c>
-      <c r="B7" s="116">
+      <c r="B7" s="2">
         <v>9605</v>
       </c>
       <c r="C7" s="53" t="s">
@@ -2711,11 +2696,11 @@
       <c r="BC7" s="14"/>
       <c r="BD7" s="51"/>
     </row>
-    <row r="8" spans="1:67" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:67" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A8" s="42">
         <v>7</v>
       </c>
-      <c r="B8" s="116">
+      <c r="B8" s="2">
         <v>9981</v>
       </c>
       <c r="C8" s="53" t="s">
@@ -2803,11 +2788,11 @@
       <c r="BC8" s="14"/>
       <c r="BD8" s="51"/>
     </row>
-    <row r="9" spans="1:67" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:67" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A9" s="42">
         <v>8</v>
       </c>
-      <c r="B9" s="116">
+      <c r="B9" s="2">
         <v>10132</v>
       </c>
       <c r="C9" s="53" t="s">
@@ -2950,11 +2935,11 @@
       <c r="BC9" s="16"/>
       <c r="BD9" s="51"/>
     </row>
-    <row r="10" spans="1:67" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:67" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="42">
         <v>9</v>
       </c>
-      <c r="B10" s="116">
+      <c r="B10" s="2">
         <v>10364</v>
       </c>
       <c r="C10" s="53" t="s">
@@ -3080,11 +3065,11 @@
       <c r="BC10" s="14"/>
       <c r="BD10" s="51"/>
     </row>
-    <row r="11" spans="1:67" ht="13.15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:67" ht="13.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="42">
         <v>10</v>
       </c>
-      <c r="B11" s="116">
+      <c r="B11" s="2">
         <v>10362</v>
       </c>
       <c r="C11" s="53" t="s">
@@ -3189,11 +3174,11 @@
       <c r="BC11" s="45"/>
       <c r="BD11" s="51"/>
     </row>
-    <row r="12" spans="1:67" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:67" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="42">
         <v>11</v>
       </c>
-      <c r="B12" s="116">
+      <c r="B12" s="2">
         <v>11275</v>
       </c>
       <c r="C12" s="53" t="s">
@@ -3314,11 +3299,11 @@
       <c r="BC12" s="16"/>
       <c r="BD12" s="51"/>
     </row>
-    <row r="13" spans="1:67" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:67" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A13" s="42">
         <v>12</v>
       </c>
-      <c r="B13" s="116">
+      <c r="B13" s="2">
         <v>11481</v>
       </c>
       <c r="C13" s="53" t="s">
@@ -3412,11 +3397,11 @@
       <c r="BC13" s="51"/>
       <c r="BD13" s="51"/>
     </row>
-    <row r="14" spans="1:67" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:67" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="42">
         <v>13</v>
       </c>
-      <c r="B14" s="116">
+      <c r="B14" s="2">
         <v>11561</v>
       </c>
       <c r="C14" s="53" t="s">
@@ -3548,11 +3533,11 @@
       <c r="BC14" s="51"/>
       <c r="BD14" s="51"/>
     </row>
-    <row r="15" spans="1:67" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:67" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="42">
         <v>14</v>
       </c>
-      <c r="B15" s="116">
+      <c r="B15" s="2">
         <v>11779</v>
       </c>
       <c r="C15" s="53" t="s">
@@ -3684,11 +3669,11 @@
       <c r="BC15" s="51"/>
       <c r="BD15" s="51"/>
     </row>
-    <row r="16" spans="1:67" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:67" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A16" s="42">
         <v>15</v>
       </c>
-      <c r="B16" s="116">
+      <c r="B16" s="2">
         <v>11847</v>
       </c>
       <c r="C16" s="53" t="s">
@@ -3776,11 +3761,11 @@
       <c r="BC16" s="51"/>
       <c r="BD16" s="51"/>
     </row>
-    <row r="17" spans="1:67" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:67" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A17" s="42">
         <v>16</v>
       </c>
-      <c r="B17" s="116">
+      <c r="B17" s="2">
         <v>11973</v>
       </c>
       <c r="C17" s="53" t="s">
@@ -3901,11 +3886,11 @@
       <c r="BC17" s="45"/>
       <c r="BD17" s="51"/>
     </row>
-    <row r="18" spans="1:67" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:67" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A18" s="42">
         <v>17</v>
       </c>
-      <c r="B18" s="116">
+      <c r="B18" s="2">
         <v>12247</v>
       </c>
       <c r="C18" s="53" t="s">
@@ -4004,11 +3989,11 @@
       <c r="BC18" s="45"/>
       <c r="BD18" s="51"/>
     </row>
-    <row r="19" spans="1:67" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:67" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A19" s="42">
         <v>18</v>
       </c>
-      <c r="B19" s="116">
+      <c r="B19" s="2">
         <v>12507</v>
       </c>
       <c r="C19" s="53" t="s">
@@ -4214,11 +4199,11 @@
       </c>
       <c r="BO19" s="48"/>
     </row>
-    <row r="20" spans="1:67" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:67" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="42">
         <v>19</v>
       </c>
-      <c r="B20" s="116">
+      <c r="B20" s="2">
         <v>12349</v>
       </c>
       <c r="C20" s="53" t="s">
@@ -4378,11 +4363,11 @@
       <c r="BC20" s="45"/>
       <c r="BD20" s="51"/>
     </row>
-    <row r="21" spans="1:67" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:67" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="42">
         <v>20</v>
       </c>
-      <c r="B21" s="116">
+      <c r="B21" s="2">
         <v>11504</v>
       </c>
       <c r="C21" s="53" t="s">
@@ -4514,11 +4499,11 @@
       <c r="BC21" s="45"/>
       <c r="BD21" s="51"/>
     </row>
-    <row r="22" spans="1:67" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:67" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A22" s="42">
         <v>21</v>
       </c>
-      <c r="B22" s="116">
+      <c r="B22" s="2">
         <v>12836</v>
       </c>
       <c r="C22" s="53" t="s">
@@ -4639,11 +4624,11 @@
       <c r="BC22" s="51"/>
       <c r="BD22" s="51"/>
     </row>
-    <row r="23" spans="1:67" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:67" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="42">
         <v>22</v>
       </c>
-      <c r="B23" s="116">
+      <c r="B23" s="2">
         <v>12845</v>
       </c>
       <c r="C23" s="53" t="s">
@@ -4805,11 +4790,11 @@
       <c r="BC23" s="51"/>
       <c r="BD23" s="51"/>
     </row>
-    <row r="24" spans="1:67" s="59" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:67" s="59" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="42">
         <v>23</v>
       </c>
-      <c r="B24" s="116">
+      <c r="B24" s="2">
         <v>12923</v>
       </c>
       <c r="C24" s="53" t="s">
@@ -4961,11 +4946,11 @@
       <c r="BC24" s="16"/>
       <c r="BD24" s="51"/>
     </row>
-    <row r="25" spans="1:67" s="59" customFormat="1" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:67" s="59" customFormat="1" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="42">
         <v>24</v>
       </c>
-      <c r="B25" s="116">
+      <c r="B25" s="2">
         <v>13207</v>
       </c>
       <c r="C25" s="53" t="s">
@@ -5074,11 +5059,11 @@
       <c r="BC25" s="51"/>
       <c r="BD25" s="51"/>
     </row>
-    <row r="26" spans="1:67" s="87" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:67" s="87" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A26" s="77">
         <v>25</v>
       </c>
-      <c r="B26" s="116">
+      <c r="B26" s="2">
         <v>13102</v>
       </c>
       <c r="C26" s="78" t="s">
@@ -5210,11 +5195,11 @@
       <c r="BC26" s="73"/>
       <c r="BD26" s="73"/>
     </row>
-    <row r="27" spans="1:67" s="59" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:67" s="59" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A27" s="42">
         <v>26</v>
       </c>
-      <c r="B27" s="116">
+      <c r="B27" s="2">
         <v>13101</v>
       </c>
       <c r="C27" s="53" t="s">
@@ -5363,11 +5348,11 @@
       <c r="BC27" s="51"/>
       <c r="BD27" s="51"/>
     </row>
-    <row r="28" spans="1:67" s="59" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:67" s="59" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A28" s="42">
         <v>27</v>
       </c>
-      <c r="B28" s="116">
+      <c r="B28" s="2">
         <v>13100</v>
       </c>
       <c r="C28" s="53" t="s">
@@ -5505,11 +5490,11 @@
       <c r="BC28" s="51"/>
       <c r="BD28" s="51"/>
     </row>
-    <row r="29" spans="1:67" s="59" customFormat="1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:67" s="59" customFormat="1" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="42">
         <v>28</v>
       </c>
-      <c r="B29" s="116">
+      <c r="B29" s="2">
         <v>13173</v>
       </c>
       <c r="C29" s="53" t="s">
@@ -5603,11 +5588,11 @@
       <c r="BC29" s="45"/>
       <c r="BD29" s="51"/>
     </row>
-    <row r="30" spans="1:67" s="59" customFormat="1" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:67" s="59" customFormat="1" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="42">
         <v>29</v>
       </c>
-      <c r="B30" s="116">
+      <c r="B30" s="2">
         <v>13414</v>
       </c>
       <c r="C30" s="53" t="s">
@@ -5701,11 +5686,11 @@
       <c r="BC30" s="51"/>
       <c r="BD30" s="51"/>
     </row>
-    <row r="31" spans="1:67" s="59" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:67" s="59" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A31" s="42">
         <v>30</v>
       </c>
-      <c r="B31" s="116">
+      <c r="B31" s="2">
         <v>13457</v>
       </c>
       <c r="C31" s="53" t="s">
@@ -5799,11 +5784,11 @@
       <c r="BC31" s="51"/>
       <c r="BD31" s="51"/>
     </row>
-    <row r="32" spans="1:67" s="59" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:67" s="59" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A32" s="42">
         <v>31</v>
       </c>
-      <c r="B32" s="116">
+      <c r="B32" s="2">
         <v>13464</v>
       </c>
       <c r="C32" s="53" t="s">
@@ -5891,11 +5876,11 @@
       <c r="BC32" s="51"/>
       <c r="BD32" s="51"/>
     </row>
-    <row r="33" spans="1:56" s="59" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:56" s="59" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="42">
         <v>32</v>
       </c>
-      <c r="B33" s="116">
+      <c r="B33" s="2">
         <v>13005</v>
       </c>
       <c r="C33" s="53" t="s">
@@ -6057,11 +6042,11 @@
       <c r="BC33" s="51"/>
       <c r="BD33" s="51"/>
     </row>
-    <row r="34" spans="1:56" s="59" customFormat="1" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:56" s="59" customFormat="1" ht="14.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="42">
         <v>33</v>
       </c>
-      <c r="B34" s="116">
+      <c r="B34" s="2">
         <v>13626</v>
       </c>
       <c r="C34" s="53" t="s">
@@ -6183,11 +6168,11 @@
       <c r="BC34" s="51"/>
       <c r="BD34" s="51"/>
     </row>
-    <row r="35" spans="1:56" s="59" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:56" s="59" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A35" s="42">
         <v>34</v>
       </c>
-      <c r="B35" s="116">
+      <c r="B35" s="2">
         <v>13625</v>
       </c>
       <c r="C35" s="53" t="s">
@@ -6283,11 +6268,11 @@
       <c r="BC35" s="51"/>
       <c r="BD35" s="51"/>
     </row>
-    <row r="36" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A36" s="42">
         <v>35</v>
       </c>
-      <c r="B36" s="116">
+      <c r="B36" s="2">
         <v>13845</v>
       </c>
       <c r="C36" s="53" t="s">
@@ -6397,11 +6382,11 @@
       <c r="BC36" s="51"/>
       <c r="BD36" s="51"/>
     </row>
-    <row r="37" spans="1:56" ht="13.9" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:56" ht="13.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="42">
         <v>36</v>
       </c>
-      <c r="B37" s="116">
+      <c r="B37" s="2">
         <v>13986</v>
       </c>
       <c r="C37" s="53" t="s">
@@ -6528,11 +6513,11 @@
       <c r="BC37" s="51"/>
       <c r="BD37" s="51"/>
     </row>
-    <row r="38" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A38" s="42">
         <v>37</v>
       </c>
-      <c r="B38" s="116">
+      <c r="B38" s="2">
         <v>13976</v>
       </c>
       <c r="C38" s="53" t="s">
@@ -6670,11 +6655,11 @@
       <c r="BC38" s="51"/>
       <c r="BD38" s="51"/>
     </row>
-    <row r="39" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A39" s="42">
         <v>38</v>
       </c>
-      <c r="B39" s="116">
+      <c r="B39" s="2">
         <v>13974</v>
       </c>
       <c r="C39" s="53" t="s">
@@ -6801,11 +6786,11 @@
       <c r="BC39" s="51"/>
       <c r="BD39" s="51"/>
     </row>
-    <row r="40" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A40" s="42">
         <v>39</v>
       </c>
-      <c r="B40" s="116">
+      <c r="B40" s="2">
         <v>13973</v>
       </c>
       <c r="C40" s="53" t="s">
@@ -6910,11 +6895,11 @@
       <c r="BC40" s="51"/>
       <c r="BD40" s="51"/>
     </row>
-    <row r="41" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A41" s="42">
         <v>40</v>
       </c>
-      <c r="B41" s="116">
+      <c r="B41" s="2">
         <v>13887</v>
       </c>
       <c r="C41" s="53" t="s">
@@ -7023,11 +7008,11 @@
       <c r="BC41" s="51"/>
       <c r="BD41" s="51"/>
     </row>
-    <row r="42" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A42" s="42">
         <v>41</v>
       </c>
-      <c r="B42" s="116">
+      <c r="B42" s="2">
         <v>13888</v>
       </c>
       <c r="C42" s="53" t="s">
@@ -7115,11 +7100,11 @@
       <c r="BC42" s="51"/>
       <c r="BD42" s="51"/>
     </row>
-    <row r="43" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A43" s="42">
         <v>42</v>
       </c>
-      <c r="B43" s="116">
+      <c r="B43" s="2">
         <v>13850</v>
       </c>
       <c r="C43" s="53" t="s">
@@ -7240,11 +7225,11 @@
       <c r="BC43" s="51"/>
       <c r="BD43" s="51"/>
     </row>
-    <row r="44" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A44" s="42">
         <v>43</v>
       </c>
-      <c r="B44" s="116">
+      <c r="B44" s="2">
         <v>13849</v>
       </c>
       <c r="C44" s="53" t="s">
@@ -7332,11 +7317,11 @@
       <c r="BC44" s="51"/>
       <c r="BD44" s="51"/>
     </row>
-    <row r="45" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A45" s="42">
         <v>44</v>
       </c>
-      <c r="B45" s="116">
+      <c r="B45" s="2">
         <v>13847</v>
       </c>
       <c r="C45" s="53" t="s">
@@ -7457,11 +7442,11 @@
       <c r="BC45" s="51"/>
       <c r="BD45" s="51"/>
     </row>
-    <row r="46" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A46" s="42">
         <v>45</v>
       </c>
-      <c r="B46" s="116">
+      <c r="B46" s="2">
         <v>13843</v>
       </c>
       <c r="C46" s="53" t="s">
@@ -7593,11 +7578,11 @@
       <c r="BC46" s="51"/>
       <c r="BD46" s="51"/>
     </row>
-    <row r="47" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A47" s="42">
         <v>46</v>
       </c>
-      <c r="B47" s="116">
+      <c r="B47" s="2">
         <v>13842</v>
       </c>
       <c r="C47" s="53" t="s">
@@ -7707,11 +7692,11 @@
       <c r="BC47" s="51"/>
       <c r="BD47" s="51"/>
     </row>
-    <row r="48" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A48" s="42">
         <v>47</v>
       </c>
-      <c r="B48" s="116">
+      <c r="B48" s="2">
         <v>13841</v>
       </c>
       <c r="C48" s="53" t="s">
@@ -7821,11 +7806,11 @@
       <c r="BC48" s="51"/>
       <c r="BD48" s="51"/>
     </row>
-    <row r="49" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A49" s="42">
         <v>48</v>
       </c>
-      <c r="B49" s="116">
+      <c r="B49" s="2">
         <v>13840</v>
       </c>
       <c r="C49" s="53" t="s">
@@ -7968,11 +7953,11 @@
       <c r="BC49" s="51"/>
       <c r="BD49" s="51"/>
     </row>
-    <row r="50" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A50" s="42">
         <v>49</v>
       </c>
-      <c r="B50" s="116">
+      <c r="B50" s="2">
         <v>13803</v>
       </c>
       <c r="C50" s="53" t="s">
@@ -8096,11 +8081,11 @@
       <c r="BC50" s="51"/>
       <c r="BD50" s="51"/>
     </row>
-    <row r="51" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A51" s="42">
         <v>50</v>
       </c>
-      <c r="B51" s="116">
+      <c r="B51" s="2">
         <v>13801</v>
       </c>
       <c r="C51" s="53" t="s">
@@ -8227,11 +8212,11 @@
       <c r="BC51" s="51"/>
       <c r="BD51" s="51"/>
     </row>
-    <row r="52" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A52" s="42">
         <v>51</v>
       </c>
-      <c r="B52" s="116">
+      <c r="B52" s="2">
         <v>13799</v>
       </c>
       <c r="C52" s="53" t="s">
@@ -8358,11 +8343,11 @@
       <c r="BC52" s="51"/>
       <c r="BD52" s="51"/>
     </row>
-    <row r="53" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A53" s="42">
         <v>52</v>
       </c>
-      <c r="B53" s="116">
+      <c r="B53" s="2">
         <v>13797</v>
       </c>
       <c r="C53" s="53" t="s">
@@ -8456,11 +8441,11 @@
       <c r="BC53" s="51"/>
       <c r="BD53" s="51"/>
     </row>
-    <row r="54" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A54" s="42">
         <v>53</v>
       </c>
-      <c r="B54" s="116">
+      <c r="B54" s="2">
         <v>13796</v>
       </c>
       <c r="C54" s="53" t="s">
@@ -8576,11 +8561,11 @@
       <c r="BC54" s="51"/>
       <c r="BD54" s="51"/>
     </row>
-    <row r="55" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A55" s="42">
         <v>54</v>
       </c>
-      <c r="B55" s="116">
+      <c r="B55" s="2">
         <v>13706</v>
       </c>
       <c r="C55" s="53" t="s">
@@ -8668,11 +8653,11 @@
       <c r="BC55" s="51"/>
       <c r="BD55" s="51"/>
     </row>
-    <row r="56" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A56" s="42">
         <v>55</v>
       </c>
-      <c r="B56" s="116">
+      <c r="B56" s="2">
         <v>13705</v>
       </c>
       <c r="C56" s="53" t="s">
@@ -8804,11 +8789,11 @@
       <c r="BC56" s="51"/>
       <c r="BD56" s="51"/>
     </row>
-    <row r="57" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A57" s="42">
         <v>56</v>
       </c>
-      <c r="B57" s="116">
+      <c r="B57" s="2">
         <v>13691</v>
       </c>
       <c r="C57" s="53" t="s">
@@ -8902,11 +8887,11 @@
       <c r="BC57" s="51"/>
       <c r="BD57" s="51"/>
     </row>
-    <row r="58" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A58" s="42">
         <v>57</v>
       </c>
-      <c r="B58" s="116">
+      <c r="B58" s="2">
         <v>13690</v>
       </c>
       <c r="C58" s="53" t="s">
@@ -9022,11 +9007,11 @@
       <c r="BC58" s="51"/>
       <c r="BD58" s="51"/>
     </row>
-    <row r="59" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A59" s="42">
         <v>58</v>
       </c>
-      <c r="B59" s="116">
+      <c r="B59" s="2">
         <v>13688</v>
       </c>
       <c r="C59" s="53" t="s">
@@ -9131,11 +9116,11 @@
       <c r="BC59" s="51"/>
       <c r="BD59" s="51"/>
     </row>
-    <row r="60" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A60" s="42">
         <v>59</v>
       </c>
-      <c r="B60" s="116">
+      <c r="B60" s="2">
         <v>13686</v>
       </c>
       <c r="C60" s="53" t="s">
@@ -9273,11 +9258,11 @@
       <c r="BC60" s="51"/>
       <c r="BD60" s="51"/>
     </row>
-    <row r="61" spans="1:56" s="100" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:56" s="100" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A61" s="88">
         <v>60</v>
       </c>
-      <c r="B61" s="116">
+      <c r="B61" s="2">
         <v>13685</v>
       </c>
       <c r="C61" s="90" t="s">
@@ -9415,11 +9400,11 @@
       <c r="BC61" s="91"/>
       <c r="BD61" s="91"/>
     </row>
-    <row r="62" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A62" s="42">
         <v>61</v>
       </c>
-      <c r="B62" s="116">
+      <c r="B62" s="2">
         <v>13595</v>
       </c>
       <c r="C62" s="53" t="s">
@@ -9541,11 +9526,11 @@
       <c r="BC62" s="51"/>
       <c r="BD62" s="51"/>
     </row>
-    <row r="63" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A63" s="42">
         <v>62</v>
       </c>
-      <c r="B63" s="116">
+      <c r="B63" s="2">
         <v>13594</v>
       </c>
       <c r="C63" s="53" t="s">
@@ -9650,11 +9635,11 @@
       <c r="BC63" s="51"/>
       <c r="BD63" s="51"/>
     </row>
-    <row r="64" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A64" s="42">
         <v>63</v>
       </c>
-      <c r="B64" s="116">
+      <c r="B64" s="2">
         <v>13519</v>
       </c>
       <c r="C64" s="53" t="s">
@@ -9764,11 +9749,11 @@
       <c r="BC64" s="51"/>
       <c r="BD64" s="51"/>
     </row>
-    <row r="65" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A65" s="42">
         <v>64</v>
       </c>
-      <c r="B65" s="116">
+      <c r="B65" s="2">
         <v>13971</v>
       </c>
       <c r="C65" s="53" t="s">
@@ -9895,11 +9880,11 @@
       <c r="BC65" s="51"/>
       <c r="BD65" s="51"/>
     </row>
-    <row r="66" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A66" s="42">
         <v>65</v>
       </c>
-      <c r="B66" s="116">
+      <c r="B66" s="2">
         <v>14044</v>
       </c>
       <c r="C66" s="53" t="s">
@@ -9998,11 +9983,11 @@
       <c r="BC66" s="51"/>
       <c r="BD66" s="51"/>
     </row>
-    <row r="67" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A67" s="42">
         <v>66</v>
       </c>
-      <c r="B67" s="116">
+      <c r="B67" s="2">
         <v>14182</v>
       </c>
       <c r="C67" s="53" t="s">
@@ -10016,7 +10001,7 @@
         <v>302.69707811900088</v>
       </c>
       <c r="F67" s="51">
-        <f t="shared" ref="F67:F130" si="18">E67/4</f>
+        <f t="shared" ref="F67:F129" si="18">E67/4</f>
         <v>75.674269529750219</v>
       </c>
       <c r="G67" s="50">
@@ -10129,11 +10114,11 @@
       <c r="BC67" s="51"/>
       <c r="BD67" s="51"/>
     </row>
-    <row r="68" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A68" s="42">
         <v>67</v>
       </c>
-      <c r="B68" s="116">
+      <c r="B68" s="2">
         <v>14183</v>
       </c>
       <c r="C68" s="53" t="s">
@@ -10143,7 +10128,7 @@
         <v>136696.67000000001</v>
       </c>
       <c r="E68" s="51">
-        <f t="shared" ref="E68:E131" si="24">D68/H68</f>
+        <f t="shared" ref="E68:E129" si="24">D68/H68</f>
         <v>281.71805209582112</v>
       </c>
       <c r="F68" s="51">
@@ -10227,11 +10212,11 @@
       <c r="BC68" s="51"/>
       <c r="BD68" s="51"/>
     </row>
-    <row r="69" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A69" s="42">
         <v>68</v>
       </c>
-      <c r="B69" s="116">
+      <c r="B69" s="2">
         <v>14184</v>
       </c>
       <c r="C69" s="53" t="s">
@@ -10325,11 +10310,11 @@
       <c r="BC69" s="51"/>
       <c r="BD69" s="51"/>
     </row>
-    <row r="70" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A70" s="42">
         <v>69</v>
       </c>
-      <c r="B70" s="116">
+      <c r="B70" s="2">
         <v>14045</v>
       </c>
       <c r="C70" s="53" t="s">
@@ -10417,11 +10402,11 @@
       <c r="BC70" s="51"/>
       <c r="BD70" s="51"/>
     </row>
-    <row r="71" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A71" s="42">
         <v>70</v>
       </c>
-      <c r="B71" s="116">
+      <c r="B71" s="2">
         <v>14140</v>
       </c>
       <c r="C71" s="53" t="s">
@@ -10526,11 +10511,11 @@
       <c r="BC71" s="51"/>
       <c r="BD71" s="51"/>
     </row>
-    <row r="72" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A72" s="42">
         <v>71</v>
       </c>
-      <c r="B72" s="116">
+      <c r="B72" s="2">
         <v>14139</v>
       </c>
       <c r="C72" s="53" t="s">
@@ -10646,11 +10631,11 @@
       <c r="BC72" s="51"/>
       <c r="BD72" s="51"/>
     </row>
-    <row r="73" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A73" s="42">
         <v>72</v>
       </c>
-      <c r="B73" s="116">
+      <c r="B73" s="2">
         <v>14138</v>
       </c>
       <c r="C73" s="53" t="s">
@@ -10777,11 +10762,11 @@
       <c r="BC73" s="51"/>
       <c r="BD73" s="51"/>
     </row>
-    <row r="74" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A74" s="42">
         <v>73</v>
       </c>
-      <c r="B74" s="116">
+      <c r="B74" s="2">
         <v>14095</v>
       </c>
       <c r="C74" s="53" t="s">
@@ -10897,11 +10882,11 @@
       <c r="BC74" s="51"/>
       <c r="BD74" s="51"/>
     </row>
-    <row r="75" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A75" s="42">
         <v>74</v>
       </c>
-      <c r="B75" s="116">
+      <c r="B75" s="2">
         <v>13848</v>
       </c>
       <c r="C75" s="78" t="s">
@@ -10989,11 +10974,11 @@
       <c r="BC75" s="51"/>
       <c r="BD75" s="51"/>
     </row>
-    <row r="76" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A76" s="42">
         <v>75</v>
       </c>
-      <c r="B76" s="116">
+      <c r="B76" s="2">
         <v>13972</v>
       </c>
       <c r="C76" s="53" t="s">
@@ -11087,11 +11072,11 @@
       <c r="BC76" s="51"/>
       <c r="BD76" s="51"/>
     </row>
-    <row r="77" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A77" s="42">
         <v>76</v>
       </c>
-      <c r="B77" s="116">
+      <c r="B77" s="2">
         <v>14052</v>
       </c>
       <c r="C77" s="53" t="s">
@@ -11190,11 +11175,11 @@
       <c r="BC77" s="51"/>
       <c r="BD77" s="51"/>
     </row>
-    <row r="78" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A78" s="42">
         <v>77</v>
       </c>
-      <c r="B78" s="116">
+      <c r="B78" s="2">
         <v>14091</v>
       </c>
       <c r="C78" s="53" t="s">
@@ -11299,11 +11284,11 @@
       <c r="BC78" s="51"/>
       <c r="BD78" s="51"/>
     </row>
-    <row r="79" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A79" s="42">
         <v>78</v>
       </c>
-      <c r="B79" s="116">
+      <c r="B79" s="2">
         <v>14094</v>
       </c>
       <c r="C79" s="53" t="s">
@@ -11419,11 +11404,11 @@
       <c r="BC79" s="51"/>
       <c r="BD79" s="51"/>
     </row>
-    <row r="80" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A80" s="42">
         <v>79</v>
       </c>
-      <c r="B80" s="116">
+      <c r="B80" s="2">
         <v>14092</v>
       </c>
       <c r="C80" s="53" t="s">
@@ -11528,11 +11513,11 @@
       <c r="BC80" s="51"/>
       <c r="BD80" s="51"/>
     </row>
-    <row r="81" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A81" s="42">
         <v>80</v>
       </c>
-      <c r="B81" s="116">
+      <c r="B81" s="2">
         <v>14270</v>
       </c>
       <c r="C81" s="53" t="s">
@@ -11648,11 +11633,11 @@
       <c r="BC81" s="51"/>
       <c r="BD81" s="51"/>
     </row>
-    <row r="82" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A82" s="42">
         <v>81</v>
       </c>
-      <c r="B82" s="116">
+      <c r="B82" s="2">
         <v>13687</v>
       </c>
       <c r="C82" s="53" t="s">
@@ -11746,11 +11731,11 @@
       <c r="BC82" s="51"/>
       <c r="BD82" s="51"/>
     </row>
-    <row r="83" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A83" s="42">
         <v>82</v>
       </c>
-      <c r="B83" s="116">
+      <c r="B83" s="2">
         <v>14386</v>
       </c>
       <c r="C83" s="53" t="s">
@@ -11838,11 +11823,11 @@
       <c r="BC83" s="14"/>
       <c r="BD83" s="51"/>
     </row>
-    <row r="84" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A84" s="42">
         <v>83</v>
       </c>
-      <c r="B84" s="116">
+      <c r="B84" s="2">
         <v>14384</v>
       </c>
       <c r="C84" s="53" t="s">
@@ -11952,11 +11937,11 @@
       <c r="BC84" s="14"/>
       <c r="BD84" s="51"/>
     </row>
-    <row r="85" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A85" s="42">
         <v>84</v>
       </c>
-      <c r="B85" s="116">
+      <c r="B85" s="2">
         <v>14387</v>
       </c>
       <c r="C85" s="53" t="s">
@@ -12050,11 +12035,11 @@
       <c r="BC85" s="14"/>
       <c r="BD85" s="51"/>
     </row>
-    <row r="86" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A86" s="42">
         <v>85</v>
       </c>
-      <c r="B86" s="116">
+      <c r="B86" s="2">
         <v>14358</v>
       </c>
       <c r="C86" s="53" t="s">
@@ -12159,11 +12144,11 @@
       <c r="BC86" s="22"/>
       <c r="BD86" s="51"/>
     </row>
-    <row r="87" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A87" s="42">
         <v>86</v>
       </c>
-      <c r="B87" s="116">
+      <c r="B87" s="2">
         <v>14383</v>
       </c>
       <c r="C87" s="53" t="s">
@@ -12251,11 +12236,11 @@
       <c r="BC87" s="14"/>
       <c r="BD87" s="51"/>
     </row>
-    <row r="88" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A88" s="42">
         <v>87</v>
       </c>
-      <c r="B88" s="116">
+      <c r="B88" s="2">
         <v>14403</v>
       </c>
       <c r="C88" s="53" t="s">
@@ -12360,11 +12345,11 @@
       <c r="BC88" s="14"/>
       <c r="BD88" s="51"/>
     </row>
-    <row r="89" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A89" s="42">
         <v>88</v>
       </c>
-      <c r="B89" s="116">
+      <c r="B89" s="2">
         <v>14440</v>
       </c>
       <c r="C89" s="53" t="s">
@@ -12496,11 +12481,11 @@
       <c r="BC89" s="14"/>
       <c r="BD89" s="51"/>
     </row>
-    <row r="90" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A90" s="42">
         <v>89</v>
       </c>
-      <c r="B90" s="116">
+      <c r="B90" s="2">
         <v>14441</v>
       </c>
       <c r="C90" s="53" t="s">
@@ -12588,11 +12573,11 @@
       <c r="BC90" s="14"/>
       <c r="BD90" s="51"/>
     </row>
-    <row r="91" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A91" s="42">
         <v>90</v>
       </c>
-      <c r="B91" s="116">
+      <c r="B91" s="2">
         <v>14442</v>
       </c>
       <c r="C91" s="53" t="s">
@@ -12702,11 +12687,11 @@
       <c r="BC91" s="51"/>
       <c r="BD91" s="51"/>
     </row>
-    <row r="92" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A92" s="42">
         <v>91</v>
       </c>
-      <c r="B92" s="116">
+      <c r="B92" s="2">
         <v>14343</v>
       </c>
       <c r="C92" s="53" t="s">
@@ -12800,11 +12785,11 @@
       <c r="BC92" s="51"/>
       <c r="BD92" s="51"/>
     </row>
-    <row r="93" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A93" s="42">
         <v>92</v>
       </c>
-      <c r="B93" s="116">
+      <c r="B93" s="2">
         <v>14342</v>
       </c>
       <c r="C93" s="53" t="s">
@@ -12920,11 +12905,11 @@
       <c r="BC93" s="51"/>
       <c r="BD93" s="51"/>
     </row>
-    <row r="94" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A94" s="42">
         <v>93</v>
       </c>
-      <c r="B94" s="116">
+      <c r="B94" s="2">
         <v>14341</v>
       </c>
       <c r="C94" s="53" t="s">
@@ -13040,11 +13025,11 @@
       <c r="BC94" s="51"/>
       <c r="BD94" s="51"/>
     </row>
-    <row r="95" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A95" s="42">
         <v>94</v>
       </c>
-      <c r="B95" s="116">
+      <c r="B95" s="2">
         <v>14340</v>
       </c>
       <c r="C95" s="53" t="s">
@@ -13138,11 +13123,11 @@
       <c r="BC95" s="51"/>
       <c r="BD95" s="51"/>
     </row>
-    <row r="96" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A96" s="42">
         <v>95</v>
       </c>
-      <c r="B96" s="116">
+      <c r="B96" s="2">
         <v>14339</v>
       </c>
       <c r="C96" s="53" t="s">
@@ -13236,11 +13221,11 @@
       <c r="BC96" s="51"/>
       <c r="BD96" s="51"/>
     </row>
-    <row r="97" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A97" s="42">
         <v>96</v>
       </c>
-      <c r="B97" s="116">
+      <c r="B97" s="2">
         <v>14338</v>
       </c>
       <c r="C97" s="53" t="s">
@@ -13345,11 +13330,11 @@
       <c r="BC97" s="51"/>
       <c r="BD97" s="51"/>
     </row>
-    <row r="98" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A98" s="42">
         <v>97</v>
       </c>
-      <c r="B98" s="116">
+      <c r="B98" s="2">
         <v>14345</v>
       </c>
       <c r="C98" s="53" t="s">
@@ -13454,11 +13439,11 @@
       <c r="BC98" s="51"/>
       <c r="BD98" s="51"/>
     </row>
-    <row r="99" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A99" s="42">
         <v>98</v>
       </c>
-      <c r="B99" s="116">
+      <c r="B99" s="2">
         <v>14346</v>
       </c>
       <c r="C99" s="53" t="s">
@@ -13563,11 +13548,11 @@
       <c r="BC99" s="51"/>
       <c r="BD99" s="51"/>
     </row>
-    <row r="100" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A100" s="42">
         <v>99</v>
       </c>
-      <c r="B100" s="116">
+      <c r="B100" s="2">
         <v>14347</v>
       </c>
       <c r="C100" s="53" t="s">
@@ -13672,11 +13657,11 @@
       <c r="BC100" s="51"/>
       <c r="BD100" s="51"/>
     </row>
-    <row r="101" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A101" s="42">
         <v>100</v>
       </c>
-      <c r="B101" s="116">
+      <c r="B101" s="2">
         <v>14348</v>
       </c>
       <c r="C101" s="53" t="s">
@@ -13781,11 +13766,11 @@
       <c r="BC101" s="51"/>
       <c r="BD101" s="51"/>
     </row>
-    <row r="102" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A102" s="42">
         <v>101</v>
       </c>
-      <c r="B102" s="116">
+      <c r="B102" s="2">
         <v>14349</v>
       </c>
       <c r="C102" s="53" t="s">
@@ -13890,11 +13875,11 @@
       <c r="BC102" s="51"/>
       <c r="BD102" s="51"/>
     </row>
-    <row r="103" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A103" s="42">
         <v>102</v>
       </c>
-      <c r="B103" s="116">
+      <c r="B103" s="2">
         <v>14350</v>
       </c>
       <c r="C103" s="53" t="s">
@@ -13999,11 +13984,11 @@
       <c r="BC103" s="51"/>
       <c r="BD103" s="51"/>
     </row>
-    <row r="104" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A104" s="42">
         <v>103</v>
       </c>
-      <c r="B104" s="116">
+      <c r="B104" s="2">
         <v>14351</v>
       </c>
       <c r="C104" s="53" t="s">
@@ -14108,11 +14093,11 @@
       <c r="BC104" s="51"/>
       <c r="BD104" s="51"/>
     </row>
-    <row r="105" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A105" s="42">
         <v>104</v>
       </c>
-      <c r="B105" s="116">
+      <c r="B105" s="2">
         <v>14352</v>
       </c>
       <c r="C105" s="53" t="s">
@@ -14206,11 +14191,11 @@
       <c r="BC105" s="51"/>
       <c r="BD105" s="51"/>
     </row>
-    <row r="106" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A106" s="42">
         <v>105</v>
       </c>
-      <c r="B106" s="116">
+      <c r="B106" s="2">
         <v>14353</v>
       </c>
       <c r="C106" s="53" t="s">
@@ -14315,11 +14300,11 @@
       <c r="BC106" s="51"/>
       <c r="BD106" s="51"/>
     </row>
-    <row r="107" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A107" s="42">
         <v>106</v>
       </c>
-      <c r="B107" s="116">
+      <c r="B107" s="2">
         <v>14354</v>
       </c>
       <c r="C107" s="53" t="s">
@@ -14413,11 +14398,11 @@
       <c r="BC107" s="51"/>
       <c r="BD107" s="51"/>
     </row>
-    <row r="108" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A108" s="42">
         <v>107</v>
       </c>
-      <c r="B108" s="116">
+      <c r="B108" s="2">
         <v>14355</v>
       </c>
       <c r="C108" s="53" t="s">
@@ -14522,11 +14507,11 @@
       <c r="BC108" s="51"/>
       <c r="BD108" s="51"/>
     </row>
-    <row r="109" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A109" s="42">
         <v>108</v>
       </c>
-      <c r="B109" s="116">
+      <c r="B109" s="2">
         <v>14356</v>
       </c>
       <c r="C109" s="53" t="s">
@@ -14631,11 +14616,11 @@
       <c r="BC109" s="51"/>
       <c r="BD109" s="51"/>
     </row>
-    <row r="110" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A110" s="42">
         <v>109</v>
       </c>
-      <c r="B110" s="116">
+      <c r="B110" s="2">
         <v>14360</v>
       </c>
       <c r="C110" s="53" t="s">
@@ -14751,11 +14736,11 @@
       <c r="BC110" s="51"/>
       <c r="BD110" s="51"/>
     </row>
-    <row r="111" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A111" s="42">
         <v>110</v>
       </c>
-      <c r="B111" s="116">
+      <c r="B111" s="2">
         <v>14361</v>
       </c>
       <c r="C111" s="53" t="s">
@@ -14860,11 +14845,11 @@
       <c r="BC111" s="51"/>
       <c r="BD111" s="51"/>
     </row>
-    <row r="112" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A112" s="42">
         <v>111</v>
       </c>
-      <c r="B112" s="116">
+      <c r="B112" s="2">
         <v>14362</v>
       </c>
       <c r="C112" s="53" t="s">
@@ -14969,11 +14954,11 @@
       <c r="BC112" s="51"/>
       <c r="BD112" s="51"/>
     </row>
-    <row r="113" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A113" s="42">
         <v>112</v>
       </c>
-      <c r="B113" s="116">
+      <c r="B113" s="2">
         <v>14363</v>
       </c>
       <c r="C113" s="53" t="s">
@@ -15078,11 +15063,11 @@
       <c r="BC113" s="51"/>
       <c r="BD113" s="51"/>
     </row>
-    <row r="114" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A114" s="42">
         <v>113</v>
       </c>
-      <c r="B114" s="116">
+      <c r="B114" s="2">
         <v>14364</v>
       </c>
       <c r="C114" s="53" t="s">
@@ -15187,11 +15172,11 @@
       <c r="BC114" s="51"/>
       <c r="BD114" s="51"/>
     </row>
-    <row r="115" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A115" s="42">
         <v>114</v>
       </c>
-      <c r="B115" s="116">
+      <c r="B115" s="2">
         <v>14530</v>
       </c>
       <c r="C115" s="53" t="s">
@@ -15285,11 +15270,11 @@
       <c r="BC115" s="51"/>
       <c r="BD115" s="51"/>
     </row>
-    <row r="116" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A116" s="42">
         <v>115</v>
       </c>
-      <c r="B116" s="116">
+      <c r="B116" s="2">
         <v>14632</v>
       </c>
       <c r="C116" s="53" t="s">
@@ -15383,11 +15368,11 @@
       <c r="BC116" s="51"/>
       <c r="BD116" s="51"/>
     </row>
-    <row r="117" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A117" s="42">
         <v>116</v>
       </c>
-      <c r="B117" s="116">
+      <c r="B117" s="2">
         <v>14640</v>
       </c>
       <c r="C117" s="53" t="s">
@@ -15481,11 +15466,11 @@
       <c r="BC117" s="51"/>
       <c r="BD117" s="51"/>
     </row>
-    <row r="118" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A118" s="42">
         <v>117</v>
       </c>
-      <c r="B118" s="116">
+      <c r="B118" s="2">
         <v>14637</v>
       </c>
       <c r="C118" s="53" t="s">
@@ -15579,11 +15564,11 @@
       <c r="BC118" s="51"/>
       <c r="BD118" s="51"/>
     </row>
-    <row r="119" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A119" s="42">
         <v>118</v>
       </c>
-      <c r="B119" s="116">
+      <c r="B119" s="2">
         <v>14634</v>
       </c>
       <c r="C119" s="53" t="s">
@@ -15677,11 +15662,11 @@
       <c r="BC119" s="51"/>
       <c r="BD119" s="51"/>
     </row>
-    <row r="120" spans="1:56" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:56" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A120" s="42">
         <v>119</v>
       </c>
-      <c r="B120" s="116">
+      <c r="B120" s="2">
         <v>14635</v>
       </c>
       <c r="C120" s="53" t="s">
@@ -15775,11 +15760,11 @@
       <c r="BC120" s="51"/>
       <c r="BD120" s="51"/>
     </row>
-    <row r="121" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A121" s="42">
         <v>120</v>
       </c>
-      <c r="B121" s="116">
+      <c r="B121" s="2">
         <v>14641</v>
       </c>
       <c r="C121" s="53" t="s">
@@ -15884,11 +15869,11 @@
       <c r="BC121" s="51"/>
       <c r="BD121" s="51"/>
     </row>
-    <row r="122" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A122" s="42">
         <v>121</v>
       </c>
-      <c r="B122" s="116">
+      <c r="B122" s="2">
         <v>14633</v>
       </c>
       <c r="C122" s="53" t="s">
@@ -15993,11 +15978,11 @@
       <c r="BC122" s="51"/>
       <c r="BD122" s="51"/>
     </row>
-    <row r="123" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A123" s="42">
         <v>122</v>
       </c>
-      <c r="B123" s="116">
+      <c r="B123" s="2">
         <v>14636</v>
       </c>
       <c r="C123" s="53" t="s">
@@ -16102,11 +16087,11 @@
       <c r="BC123" s="51"/>
       <c r="BD123" s="51"/>
     </row>
-    <row r="124" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A124" s="42">
         <v>123</v>
       </c>
-      <c r="B124" s="116">
+      <c r="B124" s="2">
         <v>14639</v>
       </c>
       <c r="C124" s="53" t="s">
@@ -16200,11 +16185,11 @@
       <c r="BC124" s="51"/>
       <c r="BD124" s="51"/>
     </row>
-    <row r="125" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A125" s="42">
         <v>124</v>
       </c>
-      <c r="B125" s="116">
+      <c r="B125" s="2">
         <v>14642</v>
       </c>
       <c r="C125" s="53" t="s">
@@ -16298,11 +16283,11 @@
       <c r="BC125" s="51"/>
       <c r="BD125" s="51"/>
     </row>
-    <row r="126" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A126" s="42">
         <v>125</v>
       </c>
-      <c r="B126" s="116">
+      <c r="B126" s="2">
         <v>14643</v>
       </c>
       <c r="C126" s="53" t="s">
@@ -16395,11 +16380,11 @@
       <c r="BC126" s="51"/>
       <c r="BD126" s="51"/>
     </row>
-    <row r="127" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A127" s="42">
         <v>126</v>
       </c>
-      <c r="B127" s="116">
+      <c r="B127" s="2">
         <v>14644</v>
       </c>
       <c r="C127" s="53" t="s">
@@ -16499,11 +16484,11 @@
       <c r="BC127" s="51"/>
       <c r="BD127" s="51"/>
     </row>
-    <row r="128" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:56" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A128" s="42">
         <v>127</v>
       </c>
-      <c r="B128" s="116">
+      <c r="B128" s="2">
         <v>14522</v>
       </c>
       <c r="C128" s="53" t="s">
@@ -16619,11 +16604,11 @@
       <c r="BC128" s="51"/>
       <c r="BD128" s="51"/>
     </row>
-    <row r="129" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:66" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A129" s="42">
         <v>128</v>
       </c>
-      <c r="B129" s="116">
+      <c r="B129" s="2">
         <v>14473</v>
       </c>
       <c r="C129" s="53" t="s">
@@ -16717,11 +16702,11 @@
       <c r="BC129" s="51"/>
       <c r="BD129" s="51"/>
     </row>
-    <row r="130" spans="1:66" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:66" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A130" s="42">
         <v>129</v>
       </c>
-      <c r="B130" s="116">
+      <c r="B130" s="2">
         <v>14439</v>
       </c>
       <c r="C130" s="53" t="s">
@@ -16820,114 +16805,114 @@
       <c r="BC130" s="51"/>
       <c r="BD130" s="51"/>
     </row>
-    <row r="131" spans="1:66" s="100" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:66" s="100" customFormat="1" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A131" s="88">
         <v>130</v>
       </c>
-      <c r="B131" s="124">
+      <c r="B131" s="121">
         <v>14382</v>
       </c>
-      <c r="C131" s="125" t="s">
+      <c r="C131" s="122" t="s">
         <v>106</v>
       </c>
-      <c r="D131" s="126">
+      <c r="D131" s="123">
         <v>76798.62</v>
       </c>
       <c r="E131" s="51"/>
       <c r="F131" s="51"/>
-      <c r="G131" s="127">
+      <c r="G131" s="124">
         <v>46155</v>
       </c>
       <c r="H131" s="70">
         <v>0</v>
       </c>
-      <c r="I131" s="124">
+      <c r="I131" s="121">
         <v>26040051</v>
       </c>
-      <c r="J131" s="128">
+      <c r="J131" s="125">
         <f t="shared" ref="J131:J151" si="29">L131+Q131+V131+AA131+AF131+AK131+AP131+AU131+AZ131+BE131+BJ131</f>
         <v>58619.5</v>
       </c>
-      <c r="K131" s="128">
+      <c r="K131" s="125">
         <f t="shared" ref="K131:K151" si="30">D131-J131</f>
         <v>18179.119999999995</v>
       </c>
-      <c r="L131" s="128">
+      <c r="L131" s="125">
         <v>27468.5</v>
       </c>
-      <c r="M131" s="129">
+      <c r="M131" s="126">
         <v>427451</v>
       </c>
-      <c r="N131" s="127">
+      <c r="N131" s="124">
         <v>46171</v>
       </c>
-      <c r="O131" s="128">
+      <c r="O131" s="125">
         <v>547.04100000000005</v>
       </c>
-      <c r="P131" s="130">
+      <c r="P131" s="127">
         <f t="shared" si="20"/>
         <v>50.212872526922112</v>
       </c>
-      <c r="Q131" s="128">
+      <c r="Q131" s="125">
         <v>31151</v>
       </c>
-      <c r="R131" s="131">
+      <c r="R131" s="128">
         <v>210921</v>
       </c>
-      <c r="S131" s="132">
+      <c r="S131" s="129">
         <v>46203</v>
       </c>
-      <c r="T131" s="128">
+      <c r="T131" s="125">
         <v>623.02229999999997</v>
       </c>
-      <c r="U131" s="130">
+      <c r="U131" s="127">
         <f t="shared" si="21"/>
         <v>49.999815415916899</v>
       </c>
-      <c r="V131" s="133"/>
-      <c r="W131" s="125"/>
-      <c r="X131" s="124"/>
-      <c r="Y131" s="128"/>
-      <c r="Z131" s="128"/>
-      <c r="AA131" s="125"/>
-      <c r="AB131" s="125"/>
-      <c r="AC131" s="125"/>
-      <c r="AD131" s="128"/>
-      <c r="AE131" s="128"/>
-      <c r="AF131" s="125"/>
-      <c r="AG131" s="125"/>
-      <c r="AH131" s="125"/>
-      <c r="AI131" s="128"/>
-      <c r="AJ131" s="128"/>
-      <c r="AK131" s="125"/>
-      <c r="AL131" s="125"/>
-      <c r="AM131" s="125"/>
-      <c r="AN131" s="128"/>
-      <c r="AO131" s="128"/>
-      <c r="AP131" s="125"/>
-      <c r="AQ131" s="125"/>
-      <c r="AR131" s="125"/>
-      <c r="AS131" s="128"/>
-      <c r="AT131" s="128"/>
-      <c r="AU131" s="125"/>
-      <c r="AV131" s="125"/>
-      <c r="AW131" s="125"/>
-      <c r="AX131" s="128"/>
-      <c r="AY131" s="128">
+      <c r="V131" s="130"/>
+      <c r="W131" s="122"/>
+      <c r="X131" s="121"/>
+      <c r="Y131" s="125"/>
+      <c r="Z131" s="125"/>
+      <c r="AA131" s="122"/>
+      <c r="AB131" s="122"/>
+      <c r="AC131" s="122"/>
+      <c r="AD131" s="125"/>
+      <c r="AE131" s="125"/>
+      <c r="AF131" s="122"/>
+      <c r="AG131" s="122"/>
+      <c r="AH131" s="122"/>
+      <c r="AI131" s="125"/>
+      <c r="AJ131" s="125"/>
+      <c r="AK131" s="122"/>
+      <c r="AL131" s="122"/>
+      <c r="AM131" s="122"/>
+      <c r="AN131" s="125"/>
+      <c r="AO131" s="125"/>
+      <c r="AP131" s="122"/>
+      <c r="AQ131" s="122"/>
+      <c r="AR131" s="122"/>
+      <c r="AS131" s="125"/>
+      <c r="AT131" s="125"/>
+      <c r="AU131" s="122"/>
+      <c r="AV131" s="122"/>
+      <c r="AW131" s="122"/>
+      <c r="AX131" s="125"/>
+      <c r="AY131" s="125">
         <f t="shared" si="27"/>
         <v>0</v>
       </c>
-      <c r="AZ131" s="134"/>
-      <c r="BA131" s="134"/>
-      <c r="BB131" s="134"/>
-      <c r="BC131" s="128"/>
-      <c r="BD131" s="128"/>
-    </row>
-    <row r="132" spans="1:66" x14ac:dyDescent="0.25">
-      <c r="A132" s="142">
+      <c r="AZ131" s="131"/>
+      <c r="BA131" s="131"/>
+      <c r="BB131" s="131"/>
+      <c r="BC131" s="125"/>
+      <c r="BD131" s="125"/>
+    </row>
+    <row r="132" spans="1:66" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A132" s="139">
         <v>131</v>
       </c>
-      <c r="B132" s="118">
+      <c r="B132" s="116">
         <v>13006</v>
       </c>
       <c r="C132" s="53" t="s">
@@ -16977,7 +16962,7 @@
       <c r="R132" s="43">
         <v>736584</v>
       </c>
-      <c r="S132" s="143">
+      <c r="S132" s="140">
         <v>46042</v>
       </c>
       <c r="T132" s="51">
@@ -17055,25 +17040,25 @@
       <c r="BM132" s="55"/>
       <c r="BN132" s="55"/>
     </row>
-    <row r="133" spans="1:66" x14ac:dyDescent="0.25">
-      <c r="A133" s="142">
+    <row r="133" spans="1:66" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A133" s="139">
         <v>132</v>
       </c>
-      <c r="B133" s="118">
+      <c r="B133" s="116">
         <v>13299</v>
       </c>
-      <c r="C133" s="119" t="s">
+      <c r="C133" s="117" t="s">
         <v>189</v>
       </c>
-      <c r="D133" s="121">
+      <c r="D133" s="119">
         <v>138451.20000000001</v>
       </c>
       <c r="E133" s="51">
-        <f t="shared" ref="E132:E151" si="35">D133/H133</f>
+        <f t="shared" ref="E133:E151" si="35">D133/H133</f>
         <v>464.37834717623855</v>
       </c>
       <c r="F133" s="51">
-        <f t="shared" ref="F131:F151" si="36">E133/4</f>
+        <f t="shared" ref="F133:F151" si="36">E133/4</f>
         <v>116.09458679405964</v>
       </c>
       <c r="G133" s="50">
@@ -17082,7 +17067,7 @@
       <c r="H133" s="70">
         <v>298.1431</v>
       </c>
-      <c r="I133" s="120">
+      <c r="I133" s="118">
         <v>12993501</v>
       </c>
       <c r="J133" s="49">
@@ -17237,17 +17222,17 @@
       <c r="BM133" s="55"/>
       <c r="BN133" s="55"/>
     </row>
-    <row r="134" spans="1:66" x14ac:dyDescent="0.25">
-      <c r="A134" s="142">
+    <row r="134" spans="1:66" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A134" s="139">
         <v>133</v>
       </c>
-      <c r="B134" s="118">
+      <c r="B134" s="116">
         <v>13319</v>
       </c>
-      <c r="C134" s="119" t="s">
+      <c r="C134" s="117" t="s">
         <v>190</v>
       </c>
-      <c r="D134" s="121">
+      <c r="D134" s="119">
         <v>419601</v>
       </c>
       <c r="E134" s="51"/>
@@ -17258,7 +17243,7 @@
       <c r="H134" s="70">
         <v>0</v>
       </c>
-      <c r="I134" s="120">
+      <c r="I134" s="118">
         <v>15775370</v>
       </c>
       <c r="J134" s="49">
@@ -17402,17 +17387,17 @@
       <c r="BM134" s="55"/>
       <c r="BN134" s="55"/>
     </row>
-    <row r="135" spans="1:66" x14ac:dyDescent="0.25">
-      <c r="A135" s="142">
+    <row r="135" spans="1:66" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A135" s="139">
         <v>134</v>
       </c>
-      <c r="B135" s="118">
+      <c r="B135" s="116">
         <v>13798</v>
       </c>
-      <c r="C135" s="119" t="s">
+      <c r="C135" s="117" t="s">
         <v>191</v>
       </c>
-      <c r="D135" s="121">
+      <c r="D135" s="119">
         <v>238144.4</v>
       </c>
       <c r="E135" s="51">
@@ -17429,7 +17414,7 @@
       <c r="H135" s="70">
         <v>446.8048</v>
       </c>
-      <c r="I135" s="120">
+      <c r="I135" s="118">
         <v>16440131</v>
       </c>
       <c r="J135" s="49">
@@ -17446,13 +17431,13 @@
       <c r="O135" s="1"/>
       <c r="P135" s="51"/>
       <c r="Q135" s="1"/>
-      <c r="R135" s="144"/>
-      <c r="S135" s="144"/>
+      <c r="R135" s="139"/>
+      <c r="S135" s="139"/>
       <c r="T135" s="6"/>
       <c r="U135" s="51"/>
       <c r="V135" s="1"/>
       <c r="W135" s="55"/>
-      <c r="X135" s="144"/>
+      <c r="X135" s="139"/>
       <c r="Y135" s="1"/>
       <c r="Z135" s="51"/>
       <c r="AA135" s="55"/>
@@ -17496,17 +17481,17 @@
       <c r="BM135" s="55"/>
       <c r="BN135" s="55"/>
     </row>
-    <row r="136" spans="1:66" x14ac:dyDescent="0.25">
-      <c r="A136" s="142">
+    <row r="136" spans="1:66" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A136" s="139">
         <v>135</v>
       </c>
-      <c r="B136" s="118">
+      <c r="B136" s="116">
         <v>14728</v>
       </c>
-      <c r="C136" s="119" t="s">
+      <c r="C136" s="117" t="s">
         <v>192</v>
       </c>
-      <c r="D136" s="121">
+      <c r="D136" s="119">
         <v>32296.42</v>
       </c>
       <c r="E136" s="51">
@@ -17523,7 +17508,7 @@
       <c r="H136" s="70">
         <v>563.28920000000005</v>
       </c>
-      <c r="I136" s="120">
+      <c r="I136" s="118">
         <v>10277666</v>
       </c>
       <c r="J136" s="49">
@@ -17568,9 +17553,9 @@
       </c>
       <c r="V136" s="55"/>
       <c r="W136" s="55"/>
-      <c r="X136" s="144"/>
+      <c r="X136" s="139"/>
       <c r="Y136" s="1"/>
-      <c r="Z136" s="144"/>
+      <c r="Z136" s="139"/>
       <c r="AA136" s="55"/>
       <c r="AB136" s="55"/>
       <c r="AC136" s="55"/>
@@ -17612,17 +17597,17 @@
       <c r="BM136" s="55"/>
       <c r="BN136" s="55"/>
     </row>
-    <row r="137" spans="1:66" x14ac:dyDescent="0.25">
-      <c r="A137" s="142">
+    <row r="137" spans="1:66" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A137" s="139">
         <v>136</v>
       </c>
-      <c r="B137" s="118">
+      <c r="B137" s="116">
         <v>14693</v>
       </c>
-      <c r="C137" s="119" t="s">
+      <c r="C137" s="117" t="s">
         <v>193</v>
       </c>
-      <c r="D137" s="121">
+      <c r="D137" s="119">
         <v>205579.51999999999</v>
       </c>
       <c r="E137" s="51"/>
@@ -17633,7 +17618,7 @@
       <c r="H137" s="70">
         <v>0</v>
       </c>
-      <c r="I137" s="120">
+      <c r="I137" s="118">
         <v>10867663</v>
       </c>
       <c r="J137" s="49">
@@ -17650,15 +17635,15 @@
       <c r="O137" s="1"/>
       <c r="P137" s="51"/>
       <c r="Q137" s="1"/>
-      <c r="R137" s="144"/>
-      <c r="S137" s="144"/>
+      <c r="R137" s="139"/>
+      <c r="S137" s="139"/>
       <c r="T137" s="6"/>
-      <c r="U137" s="144"/>
+      <c r="U137" s="139"/>
       <c r="V137" s="1"/>
       <c r="W137" s="55"/>
-      <c r="X137" s="144"/>
+      <c r="X137" s="139"/>
       <c r="Y137" s="1"/>
-      <c r="Z137" s="144"/>
+      <c r="Z137" s="139"/>
       <c r="AA137" s="55"/>
       <c r="AB137" s="55"/>
       <c r="AC137" s="55"/>
@@ -17700,17 +17685,17 @@
       <c r="BM137" s="55"/>
       <c r="BN137" s="55"/>
     </row>
-    <row r="138" spans="1:66" x14ac:dyDescent="0.25">
-      <c r="A138" s="142">
+    <row r="138" spans="1:66" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A138" s="139">
         <v>137</v>
       </c>
-      <c r="B138" s="118">
+      <c r="B138" s="116">
         <v>14851</v>
       </c>
-      <c r="C138" s="119" t="s">
+      <c r="C138" s="117" t="s">
         <v>194</v>
       </c>
-      <c r="D138" s="121">
+      <c r="D138" s="119">
         <v>90898.08</v>
       </c>
       <c r="E138" s="51">
@@ -17727,7 +17712,7 @@
       <c r="H138" s="70">
         <v>592.5163</v>
       </c>
-      <c r="I138" s="120">
+      <c r="I138" s="118">
         <v>16249183</v>
       </c>
       <c r="J138" s="49">
@@ -17755,15 +17740,15 @@
         <v>47</v>
       </c>
       <c r="Q138" s="1"/>
-      <c r="R138" s="144"/>
-      <c r="S138" s="144"/>
+      <c r="R138" s="139"/>
+      <c r="S138" s="139"/>
       <c r="T138" s="6"/>
-      <c r="U138" s="144"/>
+      <c r="U138" s="139"/>
       <c r="V138" s="1"/>
       <c r="W138" s="55"/>
-      <c r="X138" s="144"/>
+      <c r="X138" s="139"/>
       <c r="Y138" s="1"/>
-      <c r="Z138" s="144"/>
+      <c r="Z138" s="139"/>
       <c r="AA138" s="55"/>
       <c r="AB138" s="55"/>
       <c r="AC138" s="55"/>
@@ -17805,17 +17790,17 @@
       <c r="BM138" s="55"/>
       <c r="BN138" s="55"/>
     </row>
-    <row r="139" spans="1:66" x14ac:dyDescent="0.25">
-      <c r="A139" s="142">
+    <row r="139" spans="1:66" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A139" s="139">
         <v>138</v>
       </c>
-      <c r="B139" s="118">
+      <c r="B139" s="116">
         <v>14908</v>
       </c>
-      <c r="C139" s="119" t="s">
+      <c r="C139" s="117" t="s">
         <v>195</v>
       </c>
-      <c r="D139" s="121">
+      <c r="D139" s="119">
         <v>145017.53</v>
       </c>
       <c r="E139" s="51">
@@ -17832,7 +17817,7 @@
       <c r="H139" s="70">
         <v>602.33240000000001</v>
       </c>
-      <c r="I139" s="120">
+      <c r="I139" s="118">
         <v>14107157</v>
       </c>
       <c r="J139" s="49">
@@ -17860,15 +17845,15 @@
         <v>72.999706425658658</v>
       </c>
       <c r="Q139" s="1"/>
-      <c r="R139" s="144"/>
-      <c r="S139" s="144"/>
+      <c r="R139" s="139"/>
+      <c r="S139" s="139"/>
       <c r="T139" s="6"/>
-      <c r="U139" s="144"/>
+      <c r="U139" s="139"/>
       <c r="V139" s="1"/>
       <c r="W139" s="55"/>
-      <c r="X139" s="144"/>
+      <c r="X139" s="139"/>
       <c r="Y139" s="1"/>
-      <c r="Z139" s="144"/>
+      <c r="Z139" s="139"/>
       <c r="AA139" s="55"/>
       <c r="AB139" s="55"/>
       <c r="AC139" s="55"/>
@@ -17910,17 +17895,17 @@
       <c r="BM139" s="55"/>
       <c r="BN139" s="55"/>
     </row>
-    <row r="140" spans="1:66" x14ac:dyDescent="0.25">
-      <c r="A140" s="142">
+    <row r="140" spans="1:66" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A140" s="139">
         <v>139</v>
       </c>
-      <c r="B140" s="118">
+      <c r="B140" s="116">
         <v>14909</v>
       </c>
-      <c r="C140" s="119" t="s">
+      <c r="C140" s="117" t="s">
         <v>196</v>
       </c>
-      <c r="D140" s="121">
+      <c r="D140" s="119">
         <v>134872.26999999999</v>
       </c>
       <c r="E140" s="51">
@@ -17937,7 +17922,7 @@
       <c r="H140" s="70">
         <v>602.33240000000001</v>
       </c>
-      <c r="I140" s="120">
+      <c r="I140" s="118">
         <v>20327445</v>
       </c>
       <c r="J140" s="49">
@@ -17965,15 +17950,15 @@
         <v>67.999726533490261</v>
       </c>
       <c r="Q140" s="1"/>
-      <c r="R140" s="144"/>
-      <c r="S140" s="144"/>
+      <c r="R140" s="139"/>
+      <c r="S140" s="139"/>
       <c r="T140" s="6"/>
-      <c r="U140" s="144"/>
+      <c r="U140" s="139"/>
       <c r="V140" s="1"/>
       <c r="W140" s="55"/>
-      <c r="X140" s="144"/>
+      <c r="X140" s="139"/>
       <c r="Y140" s="1"/>
-      <c r="Z140" s="144"/>
+      <c r="Z140" s="139"/>
       <c r="AA140" s="55"/>
       <c r="AB140" s="55"/>
       <c r="AC140" s="55"/>
@@ -18015,17 +18000,17 @@
       <c r="BM140" s="55"/>
       <c r="BN140" s="55"/>
     </row>
-    <row r="141" spans="1:66" x14ac:dyDescent="0.25">
-      <c r="A141" s="142">
+    <row r="141" spans="1:66" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A141" s="139">
         <v>140</v>
       </c>
-      <c r="B141" s="118">
+      <c r="B141" s="116">
         <v>14956</v>
       </c>
-      <c r="C141" s="119" t="s">
+      <c r="C141" s="117" t="s">
         <v>197</v>
       </c>
-      <c r="D141" s="121">
+      <c r="D141" s="119">
         <v>93701.8</v>
       </c>
       <c r="E141" s="51">
@@ -18042,7 +18027,7 @@
       <c r="H141" s="70">
         <v>614.57749999999999</v>
       </c>
-      <c r="I141" s="120">
+      <c r="I141" s="118">
         <v>19905972</v>
       </c>
       <c r="J141" s="49">
@@ -18070,15 +18055,15 @@
         <v>46.151686084609075</v>
       </c>
       <c r="Q141" s="1"/>
-      <c r="R141" s="144"/>
-      <c r="S141" s="144"/>
+      <c r="R141" s="139"/>
+      <c r="S141" s="139"/>
       <c r="T141" s="6"/>
-      <c r="U141" s="144"/>
+      <c r="U141" s="139"/>
       <c r="V141" s="1"/>
       <c r="W141" s="55"/>
-      <c r="X141" s="144"/>
+      <c r="X141" s="139"/>
       <c r="Y141" s="1"/>
-      <c r="Z141" s="144"/>
+      <c r="Z141" s="139"/>
       <c r="AA141" s="55"/>
       <c r="AB141" s="55"/>
       <c r="AC141" s="55"/>
@@ -18120,17 +18105,17 @@
       <c r="BM141" s="55"/>
       <c r="BN141" s="55"/>
     </row>
-    <row r="142" spans="1:66" x14ac:dyDescent="0.25">
-      <c r="A142" s="142">
+    <row r="142" spans="1:66" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A142" s="139">
         <v>141</v>
       </c>
-      <c r="B142" s="118">
+      <c r="B142" s="116">
         <v>14955</v>
       </c>
-      <c r="C142" s="119" t="s">
+      <c r="C142" s="117" t="s">
         <v>198</v>
       </c>
-      <c r="D142" s="121">
+      <c r="D142" s="119">
         <v>208226.19</v>
       </c>
       <c r="E142" s="51">
@@ -18147,7 +18132,7 @@
       <c r="H142" s="70">
         <v>614.57749999999999</v>
       </c>
-      <c r="I142" s="120">
+      <c r="I142" s="118">
         <v>14061810</v>
       </c>
       <c r="J142" s="49">
@@ -18164,15 +18149,15 @@
       <c r="O142" s="1"/>
       <c r="P142" s="51"/>
       <c r="Q142" s="1"/>
-      <c r="R142" s="144"/>
-      <c r="S142" s="144"/>
+      <c r="R142" s="139"/>
+      <c r="S142" s="139"/>
       <c r="T142" s="6"/>
-      <c r="U142" s="144"/>
+      <c r="U142" s="139"/>
       <c r="V142" s="1"/>
       <c r="W142" s="55"/>
-      <c r="X142" s="144"/>
+      <c r="X142" s="139"/>
       <c r="Y142" s="1"/>
-      <c r="Z142" s="144"/>
+      <c r="Z142" s="139"/>
       <c r="AA142" s="55"/>
       <c r="AB142" s="55"/>
       <c r="AC142" s="55"/>
@@ -18214,17 +18199,17 @@
       <c r="BM142" s="55"/>
       <c r="BN142" s="55"/>
     </row>
-    <row r="143" spans="1:66" x14ac:dyDescent="0.25">
-      <c r="A143" s="142">
+    <row r="143" spans="1:66" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A143" s="139">
         <v>142</v>
       </c>
-      <c r="B143" s="118">
+      <c r="B143" s="116">
         <v>14973</v>
       </c>
-      <c r="C143" s="119" t="s">
+      <c r="C143" s="117" t="s">
         <v>199</v>
       </c>
-      <c r="D143" s="121">
+      <c r="D143" s="119">
         <v>278655.64</v>
       </c>
       <c r="E143" s="51">
@@ -18241,7 +18226,7 @@
       <c r="H143" s="70">
         <v>617.63879999999995</v>
       </c>
-      <c r="I143" s="120">
+      <c r="I143" s="118">
         <v>13517848</v>
       </c>
       <c r="J143" s="49">
@@ -18258,15 +18243,15 @@
       <c r="O143" s="1"/>
       <c r="P143" s="51"/>
       <c r="Q143" s="1"/>
-      <c r="R143" s="144"/>
-      <c r="S143" s="144"/>
+      <c r="R143" s="139"/>
+      <c r="S143" s="139"/>
       <c r="T143" s="6"/>
-      <c r="U143" s="144"/>
+      <c r="U143" s="139"/>
       <c r="V143" s="1"/>
       <c r="W143" s="55"/>
-      <c r="X143" s="144"/>
+      <c r="X143" s="139"/>
       <c r="Y143" s="1"/>
-      <c r="Z143" s="144"/>
+      <c r="Z143" s="139"/>
       <c r="AA143" s="55"/>
       <c r="AB143" s="55"/>
       <c r="AC143" s="55"/>
@@ -18308,17 +18293,17 @@
       <c r="BM143" s="55"/>
       <c r="BN143" s="55"/>
     </row>
-    <row r="144" spans="1:66" x14ac:dyDescent="0.25">
-      <c r="A144" s="142">
+    <row r="144" spans="1:66" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A144" s="139">
         <v>143</v>
       </c>
-      <c r="B144" s="118">
+      <c r="B144" s="116">
         <v>14954</v>
       </c>
-      <c r="C144" s="119" t="s">
+      <c r="C144" s="117" t="s">
         <v>200</v>
       </c>
-      <c r="D144" s="121">
+      <c r="D144" s="119">
         <v>140246.47</v>
       </c>
       <c r="E144" s="51">
@@ -18335,7 +18320,7 @@
       <c r="H144" s="70">
         <v>614.57749999999999</v>
       </c>
-      <c r="I144" s="120">
+      <c r="I144" s="118">
         <v>15466152</v>
       </c>
       <c r="J144" s="49">
@@ -18363,15 +18348,15 @@
         <v>69.227529126913623</v>
       </c>
       <c r="Q144" s="1"/>
-      <c r="R144" s="144"/>
-      <c r="S144" s="144"/>
+      <c r="R144" s="139"/>
+      <c r="S144" s="139"/>
       <c r="T144" s="6"/>
-      <c r="U144" s="144"/>
+      <c r="U144" s="139"/>
       <c r="V144" s="1"/>
       <c r="W144" s="55"/>
-      <c r="X144" s="144"/>
+      <c r="X144" s="139"/>
       <c r="Y144" s="1"/>
-      <c r="Z144" s="144"/>
+      <c r="Z144" s="139"/>
       <c r="AA144" s="55"/>
       <c r="AB144" s="55"/>
       <c r="AC144" s="55"/>
@@ -18413,17 +18398,17 @@
       <c r="BM144" s="55"/>
       <c r="BN144" s="55"/>
     </row>
-    <row r="145" spans="1:66" x14ac:dyDescent="0.25">
-      <c r="A145" s="142">
+    <row r="145" spans="1:66" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A145" s="139">
         <v>144</v>
       </c>
-      <c r="B145" s="118">
+      <c r="B145" s="116">
         <v>14971</v>
       </c>
-      <c r="C145" s="119" t="s">
+      <c r="C145" s="117" t="s">
         <v>201</v>
       </c>
-      <c r="D145" s="121">
+      <c r="D145" s="119">
         <v>200264.6</v>
       </c>
       <c r="E145" s="51">
@@ -18440,7 +18425,7 @@
       <c r="H145" s="70">
         <v>617.63879999999995</v>
       </c>
-      <c r="I145" s="120">
+      <c r="I145" s="118">
         <v>13124768</v>
       </c>
       <c r="J145" s="49">
@@ -18468,15 +18453,15 @@
         <v>97.657561495498939</v>
       </c>
       <c r="Q145" s="1"/>
-      <c r="R145" s="144"/>
-      <c r="S145" s="144"/>
+      <c r="R145" s="139"/>
+      <c r="S145" s="139"/>
       <c r="T145" s="6"/>
-      <c r="U145" s="144"/>
+      <c r="U145" s="139"/>
       <c r="V145" s="1"/>
       <c r="W145" s="55"/>
-      <c r="X145" s="144"/>
+      <c r="X145" s="139"/>
       <c r="Y145" s="1"/>
-      <c r="Z145" s="144"/>
+      <c r="Z145" s="139"/>
       <c r="AA145" s="55"/>
       <c r="AB145" s="55"/>
       <c r="AC145" s="55"/>
@@ -18518,17 +18503,17 @@
       <c r="BM145" s="55"/>
       <c r="BN145" s="55"/>
     </row>
-    <row r="146" spans="1:66" x14ac:dyDescent="0.25">
-      <c r="A146" s="142">
+    <row r="146" spans="1:66" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A146" s="139">
         <v>145</v>
       </c>
-      <c r="B146" s="118">
+      <c r="B146" s="116">
         <v>14970</v>
       </c>
-      <c r="C146" s="119" t="s">
+      <c r="C146" s="117" t="s">
         <v>202</v>
       </c>
-      <c r="D146" s="121">
+      <c r="D146" s="119">
         <v>94497.39</v>
       </c>
       <c r="E146" s="51">
@@ -18545,7 +18530,7 @@
       <c r="H146" s="70">
         <v>617.63879999999995</v>
       </c>
-      <c r="I146" s="120">
+      <c r="I146" s="118">
         <v>13165184</v>
       </c>
       <c r="J146" s="49">
@@ -18573,15 +18558,15 @@
         <v>45.83926355911175</v>
       </c>
       <c r="Q146" s="1"/>
-      <c r="R146" s="144"/>
-      <c r="S146" s="144"/>
+      <c r="R146" s="139"/>
+      <c r="S146" s="139"/>
       <c r="T146" s="6"/>
-      <c r="U146" s="144"/>
+      <c r="U146" s="139"/>
       <c r="V146" s="1"/>
       <c r="W146" s="55"/>
-      <c r="X146" s="144"/>
+      <c r="X146" s="139"/>
       <c r="Y146" s="1"/>
-      <c r="Z146" s="144"/>
+      <c r="Z146" s="139"/>
       <c r="AA146" s="55"/>
       <c r="AB146" s="55"/>
       <c r="AC146" s="55"/>
@@ -18623,17 +18608,17 @@
       <c r="BM146" s="55"/>
       <c r="BN146" s="55"/>
     </row>
-    <row r="147" spans="1:66" x14ac:dyDescent="0.25">
-      <c r="A147" s="142">
+    <row r="147" spans="1:66" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A147" s="139">
         <v>146</v>
       </c>
-      <c r="B147" s="118">
+      <c r="B147" s="116">
         <v>14972</v>
       </c>
-      <c r="C147" s="119" t="s">
+      <c r="C147" s="117" t="s">
         <v>203</v>
       </c>
-      <c r="D147" s="121">
+      <c r="D147" s="119">
         <v>14205.49</v>
       </c>
       <c r="E147" s="51">
@@ -18650,7 +18635,7 @@
       <c r="H147" s="70">
         <v>617.63879999999995</v>
       </c>
-      <c r="I147" s="120">
+      <c r="I147" s="118">
         <v>17578855</v>
       </c>
       <c r="J147" s="49">
@@ -18667,15 +18652,15 @@
       <c r="O147" s="1"/>
       <c r="P147" s="51"/>
       <c r="Q147" s="1"/>
-      <c r="R147" s="144"/>
-      <c r="S147" s="144"/>
+      <c r="R147" s="139"/>
+      <c r="S147" s="139"/>
       <c r="T147" s="6"/>
-      <c r="U147" s="144"/>
+      <c r="U147" s="139"/>
       <c r="V147" s="1"/>
       <c r="W147" s="55"/>
-      <c r="X147" s="144"/>
+      <c r="X147" s="139"/>
       <c r="Y147" s="1"/>
-      <c r="Z147" s="144"/>
+      <c r="Z147" s="139"/>
       <c r="AA147" s="55"/>
       <c r="AB147" s="55"/>
       <c r="AC147" s="55"/>
@@ -18717,17 +18702,17 @@
       <c r="BM147" s="55"/>
       <c r="BN147" s="55"/>
     </row>
-    <row r="148" spans="1:66" x14ac:dyDescent="0.25">
-      <c r="A148" s="142">
+    <row r="148" spans="1:66" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A148" s="139">
         <v>147</v>
       </c>
-      <c r="B148" s="123">
+      <c r="B148" s="41">
         <v>14357</v>
       </c>
-      <c r="C148" s="119" t="s">
+      <c r="C148" s="117" t="s">
         <v>204</v>
       </c>
-      <c r="D148" s="121">
+      <c r="D148" s="119">
         <v>28883.43</v>
       </c>
       <c r="E148" s="51">
@@ -18744,7 +18729,7 @@
       <c r="H148" s="70">
         <v>500.4606</v>
       </c>
-      <c r="I148" s="120">
+      <c r="I148" s="118">
         <v>18716174</v>
       </c>
       <c r="J148" s="49">
@@ -18761,15 +18746,15 @@
       <c r="O148" s="1"/>
       <c r="P148" s="51"/>
       <c r="Q148" s="1"/>
-      <c r="R148" s="144"/>
-      <c r="S148" s="144"/>
+      <c r="R148" s="139"/>
+      <c r="S148" s="139"/>
       <c r="T148" s="6"/>
-      <c r="U148" s="144"/>
+      <c r="U148" s="139"/>
       <c r="V148" s="1"/>
       <c r="W148" s="55"/>
-      <c r="X148" s="144"/>
+      <c r="X148" s="139"/>
       <c r="Y148" s="1"/>
-      <c r="Z148" s="144"/>
+      <c r="Z148" s="139"/>
       <c r="AA148" s="55"/>
       <c r="AB148" s="55"/>
       <c r="AC148" s="55"/>
@@ -18811,17 +18796,17 @@
       <c r="BM148" s="55"/>
       <c r="BN148" s="55"/>
     </row>
-    <row r="149" spans="1:66" x14ac:dyDescent="0.25">
-      <c r="A149" s="142">
+    <row r="149" spans="1:66" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A149" s="139">
         <v>148</v>
       </c>
-      <c r="B149" s="123">
+      <c r="B149" s="41">
         <v>14388</v>
       </c>
-      <c r="C149" s="119" t="s">
+      <c r="C149" s="117" t="s">
         <v>205</v>
       </c>
-      <c r="D149" s="121">
+      <c r="D149" s="119">
         <v>140373.6</v>
       </c>
       <c r="E149" s="51"/>
@@ -18832,7 +18817,7 @@
       <c r="H149" s="70">
         <v>0</v>
       </c>
-      <c r="I149" s="120">
+      <c r="I149" s="118">
         <v>20836764</v>
       </c>
       <c r="J149" s="49">
@@ -18849,15 +18834,15 @@
       <c r="O149" s="1"/>
       <c r="P149" s="51"/>
       <c r="Q149" s="1"/>
-      <c r="R149" s="144"/>
-      <c r="S149" s="144"/>
+      <c r="R149" s="139"/>
+      <c r="S149" s="139"/>
       <c r="T149" s="6"/>
-      <c r="U149" s="144"/>
+      <c r="U149" s="139"/>
       <c r="V149" s="1"/>
       <c r="W149" s="55"/>
-      <c r="X149" s="144"/>
+      <c r="X149" s="139"/>
       <c r="Y149" s="1"/>
-      <c r="Z149" s="144"/>
+      <c r="Z149" s="139"/>
       <c r="AA149" s="55"/>
       <c r="AB149" s="55"/>
       <c r="AC149" s="55"/>
@@ -18899,17 +18884,17 @@
       <c r="BM149" s="55"/>
       <c r="BN149" s="55"/>
     </row>
-    <row r="150" spans="1:66" x14ac:dyDescent="0.25">
-      <c r="A150" s="142">
+    <row r="150" spans="1:66" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A150" s="139">
         <v>149</v>
       </c>
-      <c r="B150" s="123">
+      <c r="B150" s="41">
         <v>14645</v>
       </c>
-      <c r="C150" s="119" t="s">
+      <c r="C150" s="117" t="s">
         <v>206</v>
       </c>
-      <c r="D150" s="121">
+      <c r="D150" s="119">
         <v>151192.5</v>
       </c>
       <c r="E150" s="51">
@@ -18926,7 +18911,7 @@
       <c r="H150" s="70">
         <v>547.04100000000005</v>
       </c>
-      <c r="I150" s="120">
+      <c r="I150" s="118">
         <v>17775169</v>
       </c>
       <c r="J150" s="49">
@@ -18943,15 +18928,15 @@
       <c r="O150" s="1"/>
       <c r="P150" s="51"/>
       <c r="Q150" s="1"/>
-      <c r="R150" s="144"/>
-      <c r="S150" s="144"/>
+      <c r="R150" s="139"/>
+      <c r="S150" s="139"/>
       <c r="T150" s="6"/>
-      <c r="U150" s="144"/>
+      <c r="U150" s="139"/>
       <c r="V150" s="1"/>
       <c r="W150" s="55"/>
-      <c r="X150" s="144"/>
+      <c r="X150" s="139"/>
       <c r="Y150" s="1"/>
-      <c r="Z150" s="144"/>
+      <c r="Z150" s="139"/>
       <c r="AA150" s="55"/>
       <c r="AB150" s="55"/>
       <c r="AC150" s="55"/>
@@ -18993,17 +18978,17 @@
       <c r="BM150" s="55"/>
       <c r="BN150" s="55"/>
     </row>
-    <row r="151" spans="1:66" x14ac:dyDescent="0.25">
-      <c r="A151" s="117">
+    <row r="151" spans="1:66" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A151" s="42">
         <v>150</v>
       </c>
-      <c r="B151" s="135">
+      <c r="B151" s="132">
         <v>14910</v>
       </c>
-      <c r="C151" s="136" t="s">
+      <c r="C151" s="133" t="s">
         <v>207</v>
       </c>
-      <c r="D151" s="137">
+      <c r="D151" s="134">
         <v>66858.63</v>
       </c>
       <c r="E151" s="51">
@@ -19014,26 +18999,26 @@
         <f t="shared" si="36"/>
         <v>27.749889429823135</v>
       </c>
-      <c r="G151" s="122">
+      <c r="G151" s="120">
         <v>46191</v>
       </c>
       <c r="H151" s="70">
         <v>602.33240000000001</v>
       </c>
-      <c r="I151" s="138">
+      <c r="I151" s="135">
         <v>20016127</v>
       </c>
-      <c r="J151" s="139">
+      <c r="J151" s="136">
         <f t="shared" si="29"/>
         <v>0</v>
       </c>
-      <c r="K151" s="139">
+      <c r="K151" s="136">
         <f t="shared" si="30"/>
         <v>66858.63</v>
       </c>
-      <c r="L151" s="140"/>
-      <c r="M151" s="141"/>
-      <c r="P151" s="140"/>
+      <c r="L151" s="137"/>
+      <c r="M151" s="138"/>
+      <c r="P151" s="137"/>
     </row>
     <row r="152" spans="1:66" x14ac:dyDescent="0.25">
       <c r="B152" s="58"/>
@@ -19041,7 +19026,7 @@
       <c r="H152" s="58"/>
     </row>
   </sheetData>
-  <autoFilter ref="B1:BO131"/>
+  <autoFilter ref="B1:BO131" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <conditionalFormatting sqref="B1:B1048576">
     <cfRule type="duplicateValues" dxfId="1" priority="1"/>
   </conditionalFormatting>
@@ -19051,252 +19036,252 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="B1:B66"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="9.5703125" style="117" customWidth="1"/>
+    <col min="2" max="2" width="9.5546875" style="42" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B1" s="118">
+    <row r="1" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B1" s="116">
         <v>13006</v>
       </c>
     </row>
-    <row r="2" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B2" s="118">
+    <row r="2" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B2" s="116">
         <v>13299</v>
       </c>
     </row>
-    <row r="3" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B3" s="118">
+    <row r="3" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B3" s="116">
         <v>13319</v>
       </c>
     </row>
-    <row r="4" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B4" s="118">
+    <row r="4" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B4" s="116">
         <v>13798</v>
       </c>
     </row>
-    <row r="5" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B5" s="118">
+    <row r="5" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B5" s="116">
         <v>13799</v>
       </c>
     </row>
-    <row r="6" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B6" s="118">
+    <row r="6" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B6" s="116">
         <v>14728</v>
       </c>
     </row>
-    <row r="7" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B7" s="118">
+    <row r="7" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B7" s="116">
         <v>14693</v>
       </c>
     </row>
-    <row r="8" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B8" s="118">
+    <row r="8" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B8" s="116">
         <v>14851</v>
       </c>
     </row>
-    <row r="9" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B9" s="118">
+    <row r="9" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B9" s="116">
         <v>14908</v>
       </c>
     </row>
-    <row r="10" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B10" s="118">
+    <row r="10" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B10" s="116">
         <v>14909</v>
       </c>
     </row>
-    <row r="11" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B11" s="118">
+    <row r="11" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B11" s="116">
         <v>14956</v>
       </c>
     </row>
-    <row r="12" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B12" s="118">
+    <row r="12" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B12" s="116">
         <v>14955</v>
       </c>
     </row>
-    <row r="13" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B13" s="118">
+    <row r="13" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B13" s="116">
         <v>14973</v>
       </c>
     </row>
-    <row r="14" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B14" s="118">
+    <row r="14" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B14" s="116">
         <v>14954</v>
       </c>
     </row>
-    <row r="15" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B15" s="118">
+    <row r="15" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B15" s="116">
         <v>14971</v>
       </c>
     </row>
-    <row r="16" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B16" s="118">
+    <row r="16" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B16" s="116">
         <v>14970</v>
       </c>
     </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B17" s="118">
+    <row r="17" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B17" s="116">
         <v>14972</v>
       </c>
     </row>
-    <row r="18" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B18" s="116"/>
-    </row>
-    <row r="19" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B19" s="116"/>
-    </row>
-    <row r="20" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B20" s="116"/>
-    </row>
-    <row r="21" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B21" s="116"/>
-    </row>
-    <row r="22" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B22" s="116"/>
-    </row>
-    <row r="23" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B23" s="116"/>
-    </row>
-    <row r="24" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B24" s="116"/>
-    </row>
-    <row r="25" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B25" s="116"/>
-    </row>
-    <row r="26" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B26" s="116"/>
-    </row>
-    <row r="27" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B27" s="116"/>
-    </row>
-    <row r="28" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B28" s="116"/>
-    </row>
-    <row r="29" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B29" s="116"/>
-    </row>
-    <row r="30" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B30" s="116"/>
-    </row>
-    <row r="31" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B31" s="116"/>
-    </row>
-    <row r="32" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B32" s="116"/>
-    </row>
-    <row r="33" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B33" s="116"/>
-    </row>
-    <row r="34" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B34" s="116"/>
-    </row>
-    <row r="35" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B35" s="116"/>
-    </row>
-    <row r="36" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B36" s="116"/>
-    </row>
-    <row r="37" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B37" s="116"/>
-    </row>
-    <row r="38" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B38" s="116"/>
-    </row>
-    <row r="39" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B39" s="116"/>
-    </row>
-    <row r="40" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B40" s="116"/>
-    </row>
-    <row r="41" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B41" s="116"/>
-    </row>
-    <row r="42" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B42" s="116"/>
-    </row>
-    <row r="43" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B43" s="116"/>
-    </row>
-    <row r="44" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B44" s="116"/>
-    </row>
-    <row r="45" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B45" s="116"/>
-    </row>
-    <row r="46" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B46" s="116"/>
-    </row>
-    <row r="47" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B47" s="116"/>
-    </row>
-    <row r="48" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B48" s="116"/>
-    </row>
-    <row r="49" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B49" s="116"/>
-    </row>
-    <row r="50" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B50" s="116"/>
-    </row>
-    <row r="51" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B51" s="116"/>
-    </row>
-    <row r="52" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B52" s="116"/>
-    </row>
-    <row r="53" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B53" s="116"/>
-    </row>
-    <row r="54" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B54" s="116"/>
-    </row>
-    <row r="55" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B55" s="116"/>
-    </row>
-    <row r="56" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B56" s="116"/>
-    </row>
-    <row r="57" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B57" s="116"/>
-    </row>
-    <row r="58" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B58" s="116"/>
-    </row>
-    <row r="59" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B59" s="116"/>
-    </row>
-    <row r="60" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B60" s="116"/>
-    </row>
-    <row r="61" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B61" s="116"/>
-    </row>
-    <row r="62" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B62" s="116"/>
-    </row>
-    <row r="63" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B63" s="116"/>
-    </row>
-    <row r="64" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B64" s="116"/>
-    </row>
-    <row r="65" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B65" s="116"/>
-    </row>
-    <row r="66" spans="2:2" x14ac:dyDescent="0.25">
-      <c r="B66" s="116"/>
+    <row r="18" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B18" s="2"/>
+    </row>
+    <row r="19" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B19" s="2"/>
+    </row>
+    <row r="20" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B20" s="2"/>
+    </row>
+    <row r="21" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B21" s="2"/>
+    </row>
+    <row r="22" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B22" s="2"/>
+    </row>
+    <row r="23" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B23" s="2"/>
+    </row>
+    <row r="24" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B24" s="2"/>
+    </row>
+    <row r="25" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B25" s="2"/>
+    </row>
+    <row r="26" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B26" s="2"/>
+    </row>
+    <row r="27" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B27" s="2"/>
+    </row>
+    <row r="28" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B28" s="2"/>
+    </row>
+    <row r="29" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B29" s="2"/>
+    </row>
+    <row r="30" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B30" s="2"/>
+    </row>
+    <row r="31" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B31" s="2"/>
+    </row>
+    <row r="32" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B32" s="2"/>
+    </row>
+    <row r="33" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B33" s="2"/>
+    </row>
+    <row r="34" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B34" s="2"/>
+    </row>
+    <row r="35" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B35" s="2"/>
+    </row>
+    <row r="36" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B36" s="2"/>
+    </row>
+    <row r="37" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B37" s="2"/>
+    </row>
+    <row r="38" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B38" s="2"/>
+    </row>
+    <row r="39" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B39" s="2"/>
+    </row>
+    <row r="40" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B40" s="2"/>
+    </row>
+    <row r="41" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B41" s="2"/>
+    </row>
+    <row r="42" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B42" s="2"/>
+    </row>
+    <row r="43" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B43" s="2"/>
+    </row>
+    <row r="44" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B44" s="2"/>
+    </row>
+    <row r="45" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B45" s="2"/>
+    </row>
+    <row r="46" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B46" s="2"/>
+    </row>
+    <row r="47" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B47" s="2"/>
+    </row>
+    <row r="48" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B48" s="2"/>
+    </row>
+    <row r="49" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B49" s="2"/>
+    </row>
+    <row r="50" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B50" s="2"/>
+    </row>
+    <row r="51" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B51" s="2"/>
+    </row>
+    <row r="52" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B52" s="2"/>
+    </row>
+    <row r="53" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B53" s="2"/>
+    </row>
+    <row r="54" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B54" s="2"/>
+    </row>
+    <row r="55" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B55" s="2"/>
+    </row>
+    <row r="56" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B56" s="2"/>
+    </row>
+    <row r="57" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B57" s="2"/>
+    </row>
+    <row r="58" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B58" s="2"/>
+    </row>
+    <row r="59" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B59" s="2"/>
+    </row>
+    <row r="60" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B60" s="2"/>
+    </row>
+    <row r="61" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B61" s="2"/>
+    </row>
+    <row r="62" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B62" s="2"/>
+    </row>
+    <row r="63" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B63" s="2"/>
+    </row>
+    <row r="64" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B64" s="2"/>
+    </row>
+    <row r="65" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B65" s="2"/>
+    </row>
+    <row r="66" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B66" s="2"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="B1:B1048576">
     <cfRule type="duplicateValues" dxfId="0" priority="1"/>
   </conditionalFormatting>
   <hyperlinks>
-    <hyperlink ref="B10" r:id="rId1" display="http://192.168.21.32/facturacion.php/fafactur/edit/id/34500"/>
-    <hyperlink ref="B14" r:id="rId2" display="http://192.168.21.32/facturacion.php/fafactur/edit/id/34559"/>
+    <hyperlink ref="B10" r:id="rId1" display="http://192.168.21.32/facturacion.php/fafactur/edit/id/34500" xr:uid="{00000000-0004-0000-0100-000000000000}"/>
+    <hyperlink ref="B14" r:id="rId2" display="http://192.168.21.32/facturacion.php/fafactur/edit/id/34559" xr:uid="{00000000-0004-0000-0100-000001000000}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>